<commit_message>
2190 - Remove percentage change formulas and totals from the template
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/_99_publication/monthly_tracker_filled_posts/templates/diagnostics_template.xlsx
+++ b/projects/_99_publication/monthly_tracker_filled_posts/templates/diagnostics_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9ABAF4C-01F6-4B76-BB20-61F211B832B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{098FF929-F05E-4B79-9C37-493ECD078187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-885" windowWidth="29040" windowHeight="15720" tabRatio="779" xr2:uid="{E876E9E8-942E-455D-9B41-2B7C7CFBA90D}"/>
   </bookViews>
@@ -241,7 +241,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -398,12 +398,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -496,6 +507,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -688,45 +700,6 @@
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="13"/>
-                <c:pt idx="0">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -833,45 +806,6 @@
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="13"/>
-                <c:pt idx="0">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -4917,45 +4851,6 @@
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="13"/>
-                <c:pt idx="0">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -5062,45 +4957,6 @@
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="13"/>
-                <c:pt idx="0">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -5471,45 +5327,6 @@
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="13"/>
-                <c:pt idx="0">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -5616,45 +5433,6 @@
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="13"/>
-                <c:pt idx="0">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -20234,14 +20012,8 @@
     </row>
     <row r="24" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B24" s="18"/>
-      <c r="C24" s="21" t="str">
-        <f>IF(SUM($E24:$G24)=0,"",SUM($E24:$G24))</f>
-        <v/>
-      </c>
-      <c r="D24" s="19" t="str">
-        <f>IF(SUM($E24:$F24)=0,"",SUM($E24:$F24))</f>
-        <v/>
-      </c>
+      <c r="C24" s="21"/>
+      <c r="D24" s="19"/>
       <c r="E24" s="19"/>
       <c r="F24" s="19"/>
       <c r="G24" s="40"/>
@@ -20272,38 +20044,17 @@
     </row>
     <row r="25" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B25" s="6"/>
-      <c r="C25" s="41" t="str">
-        <f t="shared" ref="C25:C36" si="0">IF(SUM($E25:$G25)=0,"",SUM($E25:$G25))</f>
-        <v/>
-      </c>
-      <c r="D25" s="9" t="str">
-        <f t="shared" ref="D25:D36" si="1">IF(SUM($E25:$F25)=0,"",SUM($E25:$F25))</f>
-        <v/>
-      </c>
+      <c r="C25" s="41"/>
+      <c r="D25" s="9"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
       <c r="G25" s="10"/>
       <c r="I25" s="6"/>
-      <c r="J25" s="28" t="str">
-        <f>IFERROR((C25-C24)/C24,"")</f>
-        <v/>
-      </c>
-      <c r="K25" s="3" t="str">
-        <f t="shared" ref="K25:K36" si="2">IFERROR((D25-D24)/D24,"")</f>
-        <v/>
-      </c>
-      <c r="L25" s="3" t="str">
-        <f>IF(E25="","",IFERROR((E25-E24)/E24,""))</f>
-        <v/>
-      </c>
-      <c r="M25" s="3" t="str">
-        <f t="shared" ref="M25:N25" si="3">IF(F25="","",IFERROR((F25-F24)/F24,""))</f>
-        <v/>
-      </c>
-      <c r="N25" s="29" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="J25" s="28"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="29"/>
       <c r="P25" s="6"/>
       <c r="Q25" s="8"/>
       <c r="R25" s="8"/>
@@ -20325,38 +20076,17 @@
     </row>
     <row r="26" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B26" s="6"/>
-      <c r="C26" s="41" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D26" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="C26" s="41"/>
+      <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
       <c r="G26" s="10"/>
       <c r="I26" s="6"/>
-      <c r="J26" s="28" t="str">
-        <f t="shared" ref="J26:J36" si="4">IFERROR((C26-C25)/C25,"")</f>
-        <v/>
-      </c>
-      <c r="K26" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L26" s="3" t="str">
-        <f t="shared" ref="L26:L36" si="5">IF(E26="","",IFERROR((E26-E25)/E25,""))</f>
-        <v/>
-      </c>
-      <c r="M26" s="3" t="str">
-        <f t="shared" ref="M26:M36" si="6">IF(F26="","",IFERROR((F26-F25)/F25,""))</f>
-        <v/>
-      </c>
-      <c r="N26" s="29" t="str">
-        <f t="shared" ref="N26:N36" si="7">IF(G26="","",IFERROR((G26-G25)/G25,""))</f>
-        <v/>
-      </c>
+      <c r="J26" s="28"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="29"/>
       <c r="P26" s="6"/>
       <c r="Q26" s="8"/>
       <c r="R26" s="8"/>
@@ -20379,38 +20109,17 @@
     </row>
     <row r="27" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B27" s="6"/>
-      <c r="C27" s="41" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D27" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="C27" s="41"/>
+      <c r="D27" s="9"/>
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
       <c r="G27" s="10"/>
       <c r="I27" s="6"/>
-      <c r="J27" s="28" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K27" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L27" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="M27" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="N27" s="29" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
+      <c r="J27" s="28"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="29"/>
       <c r="P27" s="6"/>
       <c r="Q27" s="8"/>
       <c r="R27" s="8"/>
@@ -20435,38 +20144,17 @@
     </row>
     <row r="28" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B28" s="6"/>
-      <c r="C28" s="41" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D28" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="C28" s="41"/>
+      <c r="D28" s="9"/>
       <c r="E28" s="9"/>
       <c r="F28" s="9"/>
       <c r="G28" s="10"/>
       <c r="I28" s="6"/>
-      <c r="J28" s="28" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K28" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L28" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="M28" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="N28" s="29" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
+      <c r="J28" s="28"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="29"/>
       <c r="P28" s="6"/>
       <c r="Q28" s="8"/>
       <c r="R28" s="8"/>
@@ -20491,38 +20179,17 @@
     </row>
     <row r="29" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B29" s="6"/>
-      <c r="C29" s="41" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D29" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="C29" s="41"/>
+      <c r="D29" s="9"/>
       <c r="E29" s="9"/>
       <c r="F29" s="9"/>
       <c r="G29" s="10"/>
       <c r="I29" s="6"/>
-      <c r="J29" s="28" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K29" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L29" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="M29" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="N29" s="29" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
+      <c r="J29" s="28"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="3"/>
+      <c r="N29" s="29"/>
       <c r="P29" s="6"/>
       <c r="Q29" s="8"/>
       <c r="R29" s="8"/>
@@ -20547,38 +20214,17 @@
     </row>
     <row r="30" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B30" s="6"/>
-      <c r="C30" s="41" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D30" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="C30" s="41"/>
+      <c r="D30" s="9"/>
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
       <c r="G30" s="10"/>
       <c r="I30" s="6"/>
-      <c r="J30" s="28" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K30" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L30" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="M30" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="N30" s="29" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
+      <c r="J30" s="28"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+      <c r="N30" s="29"/>
       <c r="P30" s="6"/>
       <c r="Q30" s="8"/>
       <c r="R30" s="8"/>
@@ -20603,38 +20249,17 @@
     </row>
     <row r="31" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B31" s="6"/>
-      <c r="C31" s="41" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D31" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="C31" s="41"/>
+      <c r="D31" s="9"/>
       <c r="E31" s="9"/>
       <c r="F31" s="9"/>
       <c r="G31" s="10"/>
       <c r="I31" s="6"/>
-      <c r="J31" s="28" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K31" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L31" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="M31" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="N31" s="29" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
+      <c r="J31" s="28"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="3"/>
+      <c r="N31" s="29"/>
       <c r="Q31" s="8"/>
       <c r="R31" s="8"/>
       <c r="S31" s="8"/>
@@ -20654,38 +20279,17 @@
     </row>
     <row r="32" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B32" s="6"/>
-      <c r="C32" s="41" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D32" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="C32" s="41"/>
+      <c r="D32" s="9"/>
       <c r="E32" s="9"/>
       <c r="F32" s="9"/>
       <c r="G32" s="10"/>
       <c r="I32" s="6"/>
-      <c r="J32" s="28" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K32" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L32" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="M32" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="N32" s="29" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
+      <c r="J32" s="28"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="3"/>
+      <c r="N32" s="29"/>
       <c r="Q32" s="8"/>
       <c r="R32" s="8"/>
       <c r="S32" s="8"/>
@@ -20705,38 +20309,17 @@
     </row>
     <row r="33" spans="2:36" x14ac:dyDescent="0.2">
       <c r="B33" s="6"/>
-      <c r="C33" s="41" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D33" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="C33" s="41"/>
+      <c r="D33" s="9"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="10"/>
       <c r="I33" s="6"/>
-      <c r="J33" s="28" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K33" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L33" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="M33" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="N33" s="29" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
+      <c r="J33" s="28"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
+      <c r="N33" s="29"/>
       <c r="Q33" s="8"/>
       <c r="R33" s="8"/>
       <c r="S33" s="8"/>
@@ -20755,38 +20338,17 @@
     </row>
     <row r="34" spans="2:36" x14ac:dyDescent="0.2">
       <c r="B34" s="6"/>
-      <c r="C34" s="41" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D34" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="C34" s="41"/>
+      <c r="D34" s="9"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="10"/>
       <c r="I34" s="6"/>
-      <c r="J34" s="28" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K34" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L34" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="M34" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="N34" s="29" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
+      <c r="J34" s="28"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
+      <c r="N34" s="29"/>
       <c r="Q34" s="8"/>
       <c r="R34" s="8"/>
       <c r="S34" s="8"/>
@@ -20805,38 +20367,17 @@
     </row>
     <row r="35" spans="2:36" x14ac:dyDescent="0.2">
       <c r="B35" s="6"/>
-      <c r="C35" s="41" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D35" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="C35" s="41"/>
+      <c r="D35" s="9"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="10"/>
       <c r="I35" s="6"/>
-      <c r="J35" s="28" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K35" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L35" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="M35" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="N35" s="29" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
+      <c r="J35" s="28"/>
+      <c r="K35" s="3"/>
+      <c r="L35" s="3"/>
+      <c r="M35" s="3"/>
+      <c r="N35" s="29"/>
       <c r="Q35" s="8"/>
       <c r="R35" s="8"/>
       <c r="S35" s="8"/>
@@ -20855,38 +20396,17 @@
     </row>
     <row r="36" spans="2:36" x14ac:dyDescent="0.2">
       <c r="B36" s="6"/>
-      <c r="C36" s="41" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D36" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="C36" s="41"/>
+      <c r="D36" s="9"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="10"/>
       <c r="I36" s="6"/>
-      <c r="J36" s="28" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K36" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L36" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="M36" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="N36" s="29" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
+      <c r="J36" s="28"/>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="3"/>
+      <c r="N36" s="29"/>
       <c r="Q36" s="8"/>
       <c r="R36" s="8"/>
       <c r="S36" s="8"/>
@@ -21038,14 +20558,8 @@
     </row>
     <row r="44" spans="2:36" s="33" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B44" s="18"/>
-      <c r="C44" s="21" t="str">
-        <f>IF(SUM($E44:$G44)=0,"",SUM($E44:$G44))</f>
-        <v/>
-      </c>
-      <c r="D44" s="19" t="str">
-        <f>IF(SUM($E44:$F44)=0,"",SUM($E44:$F44))</f>
-        <v/>
-      </c>
+      <c r="C44" s="21"/>
+      <c r="D44" s="19"/>
       <c r="E44" s="19"/>
       <c r="F44" s="19"/>
       <c r="G44" s="40"/>
@@ -21059,326 +20573,137 @@
     </row>
     <row r="45" spans="2:36" s="33" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B45" s="6"/>
-      <c r="C45" s="41" t="str">
-        <f t="shared" ref="C45:C56" si="8">IF(SUM($E45:$G45)=0,"",SUM($E45:$G45))</f>
-        <v/>
-      </c>
-      <c r="D45" s="9" t="str">
-        <f t="shared" ref="D45:D56" si="9">IF(SUM($E45:$F45)=0,"",SUM($E45:$F45))</f>
-        <v/>
-      </c>
+      <c r="C45" s="41"/>
+      <c r="D45" s="9"/>
       <c r="E45" s="9"/>
       <c r="F45" s="9"/>
       <c r="G45" s="10"/>
       <c r="H45" s="1"/>
       <c r="I45" s="6"/>
-      <c r="J45" s="28" t="str">
-        <f>IFERROR((C45-C44)/C44,"")</f>
-        <v/>
-      </c>
-      <c r="K45" s="3" t="str">
-        <f t="shared" ref="K45:K56" si="10">IFERROR((D45-D44)/D44,"")</f>
-        <v/>
-      </c>
-      <c r="L45" s="3" t="str">
-        <f>IF(E45="","",IFERROR((E45-E44)/E44,""))</f>
-        <v/>
-      </c>
-      <c r="M45" s="3" t="str">
-        <f t="shared" ref="M45:N45" si="11">IF(F45="","",IFERROR((F45-F44)/F44,""))</f>
-        <v/>
-      </c>
-      <c r="N45" s="29" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
+      <c r="J45" s="28"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
+      <c r="N45" s="29"/>
     </row>
     <row r="46" spans="2:36" s="33" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B46" s="6"/>
-      <c r="C46" s="41" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="D46" s="9" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
+      <c r="C46" s="41"/>
+      <c r="D46" s="9"/>
       <c r="E46" s="9"/>
       <c r="F46" s="9"/>
       <c r="G46" s="10"/>
       <c r="H46" s="1"/>
       <c r="I46" s="6"/>
-      <c r="J46" s="28" t="str">
-        <f t="shared" ref="J46:J56" si="12">IFERROR((C46-C45)/C45,"")</f>
-        <v/>
-      </c>
-      <c r="K46" s="3" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="L46" s="3" t="str">
-        <f t="shared" ref="L46:L56" si="13">IF(E46="","",IFERROR((E46-E45)/E45,""))</f>
-        <v/>
-      </c>
-      <c r="M46" s="3" t="str">
-        <f t="shared" ref="M46:M56" si="14">IF(F46="","",IFERROR((F46-F45)/F45,""))</f>
-        <v/>
-      </c>
-      <c r="N46" s="29" t="str">
-        <f t="shared" ref="N46:N56" si="15">IF(G46="","",IFERROR((G46-G45)/G45,""))</f>
-        <v/>
-      </c>
+      <c r="J46" s="28"/>
+      <c r="K46" s="3"/>
+      <c r="L46" s="3"/>
+      <c r="M46" s="3"/>
+      <c r="N46" s="29"/>
     </row>
     <row r="47" spans="2:36" s="33" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B47" s="6"/>
-      <c r="C47" s="41" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="D47" s="9" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
+      <c r="C47" s="41"/>
+      <c r="D47" s="9"/>
       <c r="E47" s="9"/>
       <c r="F47" s="9"/>
       <c r="G47" s="10"/>
       <c r="H47" s="1"/>
       <c r="I47" s="6"/>
-      <c r="J47" s="28" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="K47" s="3" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="L47" s="3" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="M47" s="3" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="N47" s="29" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
+      <c r="J47" s="28"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="3"/>
+      <c r="M47" s="3"/>
+      <c r="N47" s="29"/>
     </row>
     <row r="48" spans="2:36" s="33" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B48" s="6"/>
-      <c r="C48" s="41" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="D48" s="9" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
+      <c r="C48" s="41"/>
+      <c r="D48" s="9"/>
       <c r="E48" s="9"/>
       <c r="F48" s="9"/>
       <c r="G48" s="10"/>
       <c r="H48" s="1"/>
       <c r="I48" s="6"/>
-      <c r="J48" s="28" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="K48" s="3" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="L48" s="3" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="M48" s="3" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="N48" s="29" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
+      <c r="J48" s="28"/>
+      <c r="K48" s="3"/>
+      <c r="L48" s="3"/>
+      <c r="M48" s="3"/>
+      <c r="N48" s="29"/>
     </row>
     <row r="49" spans="2:36" s="33" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B49" s="6"/>
-      <c r="C49" s="41" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="D49" s="9" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
+      <c r="C49" s="41"/>
+      <c r="D49" s="9"/>
       <c r="E49" s="9"/>
       <c r="F49" s="9"/>
       <c r="G49" s="10"/>
       <c r="H49" s="1"/>
       <c r="I49" s="6"/>
-      <c r="J49" s="28" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="K49" s="3" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="L49" s="3" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="M49" s="3" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="N49" s="29" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
+      <c r="J49" s="28"/>
+      <c r="K49" s="3"/>
+      <c r="L49" s="3"/>
+      <c r="M49" s="3"/>
+      <c r="N49" s="29"/>
     </row>
     <row r="50" spans="2:36" s="33" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B50" s="6"/>
-      <c r="C50" s="41" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="D50" s="9" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
+      <c r="C50" s="41"/>
+      <c r="D50" s="9"/>
       <c r="E50" s="9"/>
       <c r="F50" s="9"/>
       <c r="G50" s="10"/>
       <c r="H50" s="1"/>
       <c r="I50" s="6"/>
-      <c r="J50" s="28" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="K50" s="3" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="L50" s="3" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="M50" s="3" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="N50" s="29" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
+      <c r="J50" s="28"/>
+      <c r="K50" s="3"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="3"/>
+      <c r="N50" s="29"/>
     </row>
     <row r="51" spans="2:36" s="33" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B51" s="6"/>
-      <c r="C51" s="41" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="D51" s="9" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
+      <c r="C51" s="41"/>
+      <c r="D51" s="9"/>
       <c r="E51" s="9"/>
       <c r="F51" s="9"/>
       <c r="G51" s="10"/>
       <c r="H51" s="1"/>
       <c r="I51" s="6"/>
-      <c r="J51" s="28" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="K51" s="3" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="L51" s="3" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="M51" s="3" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="N51" s="29" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
+      <c r="J51" s="28"/>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
+      <c r="N51" s="29"/>
     </row>
     <row r="52" spans="2:36" s="33" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B52" s="6"/>
-      <c r="C52" s="41" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="D52" s="9" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
+      <c r="C52" s="41"/>
+      <c r="D52" s="9"/>
       <c r="E52" s="9"/>
       <c r="F52" s="9"/>
       <c r="G52" s="10"/>
       <c r="H52" s="1"/>
       <c r="I52" s="6"/>
-      <c r="J52" s="28" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="K52" s="3" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="L52" s="3" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="M52" s="3" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="N52" s="29" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
+      <c r="J52" s="28"/>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+      <c r="M52" s="3"/>
+      <c r="N52" s="29"/>
     </row>
     <row r="53" spans="2:36" x14ac:dyDescent="0.2">
       <c r="B53" s="6"/>
-      <c r="C53" s="41" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="D53" s="9" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
+      <c r="C53" s="41"/>
+      <c r="D53" s="9"/>
       <c r="E53" s="9"/>
       <c r="F53" s="9"/>
       <c r="G53" s="10"/>
       <c r="I53" s="6"/>
-      <c r="J53" s="28" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="K53" s="3" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="L53" s="3" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="M53" s="3" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="N53" s="29" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
+      <c r="J53" s="28"/>
+      <c r="K53" s="3"/>
+      <c r="L53" s="3"/>
+      <c r="M53" s="3"/>
+      <c r="N53" s="29"/>
       <c r="Q53" s="8"/>
       <c r="R53" s="8"/>
       <c r="S53" s="8"/>
@@ -21397,38 +20722,17 @@
     </row>
     <row r="54" spans="2:36" x14ac:dyDescent="0.2">
       <c r="B54" s="6"/>
-      <c r="C54" s="41" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="D54" s="9" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
+      <c r="C54" s="41"/>
+      <c r="D54" s="9"/>
       <c r="E54" s="9"/>
       <c r="F54" s="9"/>
       <c r="G54" s="10"/>
       <c r="I54" s="6"/>
-      <c r="J54" s="28" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="K54" s="3" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="L54" s="3" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="M54" s="3" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="N54" s="29" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
+      <c r="J54" s="28"/>
+      <c r="K54" s="3"/>
+      <c r="L54" s="3"/>
+      <c r="M54" s="3"/>
+      <c r="N54" s="29"/>
       <c r="Q54" s="8"/>
       <c r="R54" s="8"/>
       <c r="S54" s="8"/>
@@ -21447,38 +20751,17 @@
     </row>
     <row r="55" spans="2:36" x14ac:dyDescent="0.2">
       <c r="B55" s="6"/>
-      <c r="C55" s="41" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="D55" s="9" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
+      <c r="C55" s="41"/>
+      <c r="D55" s="9"/>
       <c r="E55" s="9"/>
       <c r="F55" s="9"/>
       <c r="G55" s="10"/>
       <c r="I55" s="6"/>
-      <c r="J55" s="28" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="K55" s="3" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="L55" s="3" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="M55" s="3" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="N55" s="29" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
+      <c r="J55" s="28"/>
+      <c r="K55" s="3"/>
+      <c r="L55" s="3"/>
+      <c r="M55" s="3"/>
+      <c r="N55" s="29"/>
       <c r="Q55" s="8"/>
       <c r="R55" s="8"/>
       <c r="S55" s="8"/>
@@ -21497,38 +20780,17 @@
     </row>
     <row r="56" spans="2:36" x14ac:dyDescent="0.2">
       <c r="B56" s="6"/>
-      <c r="C56" s="41" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="D56" s="9" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
+      <c r="C56" s="41"/>
+      <c r="D56" s="9"/>
       <c r="E56" s="9"/>
       <c r="F56" s="9"/>
       <c r="G56" s="10"/>
       <c r="I56" s="6"/>
-      <c r="J56" s="28" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="K56" s="3" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="L56" s="3" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="M56" s="3" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="N56" s="29" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
+      <c r="J56" s="28"/>
+      <c r="K56" s="3"/>
+      <c r="L56" s="3"/>
+      <c r="M56" s="3"/>
+      <c r="N56" s="29"/>
       <c r="Q56" s="8"/>
       <c r="R56" s="8"/>
       <c r="S56" s="8"/>
@@ -21644,38 +20906,17 @@
     </row>
     <row r="65" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B65" s="6"/>
-      <c r="C65" s="41" t="str">
-        <f>IF(SUM($E65:$G65)=0,"",SUM($E65:$G65))</f>
-        <v/>
-      </c>
-      <c r="D65" s="9" t="str">
-        <f>IF(SUM($E65:$F65)=0,"",SUM($E65:$F65))</f>
-        <v/>
-      </c>
+      <c r="C65" s="41"/>
+      <c r="D65" s="9"/>
       <c r="E65" s="9"/>
       <c r="F65" s="9"/>
       <c r="G65" s="10"/>
       <c r="I65" s="6"/>
-      <c r="J65" s="28" t="e">
-        <f>IFERROR((C65-C$65)/C$65,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K65" s="3" t="e">
-        <f>IFERROR((D65-D$65)/D$65,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="L65" s="3" t="e">
-        <f>IF(E65="",NA(),IFERROR((E65-E$65)/E$65,NA()))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="M65" s="3" t="e">
-        <f t="shared" ref="M65:N65" si="16">IF(F65="",NA(),IFERROR((F65-F$65)/F$65,NA()))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="N65" s="29" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J65" s="28"/>
+      <c r="K65" s="3"/>
+      <c r="L65" s="3"/>
+      <c r="M65" s="3"/>
+      <c r="N65" s="29"/>
       <c r="P65" s="6"/>
       <c r="Q65" s="8"/>
       <c r="R65" s="8"/>
@@ -21694,38 +20935,17 @@
     </row>
     <row r="66" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B66" s="6"/>
-      <c r="C66" s="41" t="str">
-        <f t="shared" ref="C66:C77" si="17">IF(SUM($E66:$G66)=0,"",SUM($E66:$G66))</f>
-        <v/>
-      </c>
-      <c r="D66" s="9" t="str">
-        <f t="shared" ref="D66:D77" si="18">IF(SUM($E66:$F66)=0,"",SUM($E66:$F66))</f>
-        <v/>
-      </c>
+      <c r="C66" s="41"/>
+      <c r="D66" s="9"/>
       <c r="E66" s="9"/>
       <c r="F66" s="9"/>
       <c r="G66" s="10"/>
       <c r="I66" s="6"/>
-      <c r="J66" s="28" t="e">
-        <f>IFERROR((C66-C$65)/C$65,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K66" s="3" t="e">
-        <f t="shared" ref="K66" si="19">IFERROR((D66-D$65)/D$65,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="L66" s="3" t="e">
-        <f t="shared" ref="L66:L77" si="20">IF(E66="",NA(),IFERROR((E66-E$65)/E$65,NA()))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="M66" s="3" t="e">
-        <f t="shared" ref="M66:M77" si="21">IF(F66="",NA(),IFERROR((F66-F$65)/F$65,NA()))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="N66" s="29" t="e">
-        <f t="shared" ref="N66:N77" si="22">IF(G66="",NA(),IFERROR((G66-G$65)/G$65,NA()))</f>
-        <v>#N/A</v>
-      </c>
+      <c r="J66" s="28"/>
+      <c r="K66" s="3"/>
+      <c r="L66" s="3"/>
+      <c r="M66" s="3"/>
+      <c r="N66" s="29"/>
       <c r="P66" s="6"/>
       <c r="Q66" s="8"/>
       <c r="R66" s="8"/>
@@ -21744,38 +20964,17 @@
     </row>
     <row r="67" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B67" s="6"/>
-      <c r="C67" s="41" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="D67" s="9" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
+      <c r="C67" s="41"/>
+      <c r="D67" s="9"/>
       <c r="E67" s="9"/>
       <c r="F67" s="9"/>
       <c r="G67" s="10"/>
       <c r="I67" s="6"/>
-      <c r="J67" s="28" t="e">
-        <f t="shared" ref="J67:J77" si="23">IFERROR((C67-C$65)/C$65,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K67" s="3" t="e">
-        <f t="shared" ref="K67:K77" si="24">IFERROR((D67-D$65)/D$65,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="L67" s="3" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M67" s="3" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N67" s="29" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J67" s="28"/>
+      <c r="K67" s="3"/>
+      <c r="L67" s="3"/>
+      <c r="M67" s="3"/>
+      <c r="N67" s="29"/>
       <c r="P67" s="6"/>
       <c r="Q67" s="8"/>
       <c r="R67" s="8"/>
@@ -21792,38 +20991,17 @@
     </row>
     <row r="68" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B68" s="6"/>
-      <c r="C68" s="41" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="D68" s="9" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
+      <c r="C68" s="41"/>
+      <c r="D68" s="9"/>
       <c r="E68" s="9"/>
       <c r="F68" s="9"/>
       <c r="G68" s="10"/>
       <c r="I68" s="6"/>
-      <c r="J68" s="28" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K68" s="3" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L68" s="3" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M68" s="3" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N68" s="29" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J68" s="28"/>
+      <c r="K68" s="3"/>
+      <c r="L68" s="3"/>
+      <c r="M68" s="3"/>
+      <c r="N68" s="29"/>
       <c r="P68" s="6"/>
       <c r="Q68" s="8"/>
       <c r="R68" s="8"/>
@@ -21840,38 +21018,17 @@
     </row>
     <row r="69" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B69" s="6"/>
-      <c r="C69" s="41" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="D69" s="9" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
+      <c r="C69" s="41"/>
+      <c r="D69" s="9"/>
       <c r="E69" s="9"/>
       <c r="F69" s="9"/>
       <c r="G69" s="10"/>
       <c r="I69" s="6"/>
-      <c r="J69" s="28" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K69" s="3" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L69" s="3" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M69" s="3" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N69" s="29" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J69" s="28"/>
+      <c r="K69" s="3"/>
+      <c r="L69" s="3"/>
+      <c r="M69" s="3"/>
+      <c r="N69" s="29"/>
       <c r="P69" s="6"/>
       <c r="Q69" s="8"/>
       <c r="R69" s="8"/>
@@ -21888,38 +21045,17 @@
     </row>
     <row r="70" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B70" s="6"/>
-      <c r="C70" s="41" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="D70" s="9" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
+      <c r="C70" s="41"/>
+      <c r="D70" s="9"/>
       <c r="E70" s="9"/>
       <c r="F70" s="9"/>
       <c r="G70" s="10"/>
       <c r="I70" s="6"/>
-      <c r="J70" s="28" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K70" s="3" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L70" s="3" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M70" s="3" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N70" s="29" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J70" s="28"/>
+      <c r="K70" s="3"/>
+      <c r="L70" s="3"/>
+      <c r="M70" s="3"/>
+      <c r="N70" s="29"/>
       <c r="P70" s="6"/>
       <c r="Q70" s="8"/>
       <c r="R70" s="8"/>
@@ -21936,38 +21072,17 @@
     </row>
     <row r="71" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B71" s="6"/>
-      <c r="C71" s="41" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="D71" s="9" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
+      <c r="C71" s="41"/>
+      <c r="D71" s="9"/>
       <c r="E71" s="9"/>
       <c r="F71" s="9"/>
       <c r="G71" s="10"/>
       <c r="I71" s="6"/>
-      <c r="J71" s="28" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K71" s="3" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L71" s="3" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M71" s="3" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N71" s="29" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J71" s="28"/>
+      <c r="K71" s="3"/>
+      <c r="L71" s="3"/>
+      <c r="M71" s="3"/>
+      <c r="N71" s="29"/>
       <c r="P71" s="6"/>
       <c r="Q71" s="8"/>
       <c r="R71" s="8"/>
@@ -21984,38 +21099,17 @@
     </row>
     <row r="72" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B72" s="6"/>
-      <c r="C72" s="41" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="D72" s="9" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
+      <c r="C72" s="41"/>
+      <c r="D72" s="9"/>
       <c r="E72" s="9"/>
       <c r="F72" s="9"/>
       <c r="G72" s="10"/>
       <c r="I72" s="6"/>
-      <c r="J72" s="28" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K72" s="3" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L72" s="3" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M72" s="3" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N72" s="29" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J72" s="28"/>
+      <c r="K72" s="3"/>
+      <c r="L72" s="3"/>
+      <c r="M72" s="3"/>
+      <c r="N72" s="29"/>
       <c r="P72" s="6"/>
       <c r="Q72" s="8"/>
       <c r="R72" s="8"/>
@@ -22032,38 +21126,17 @@
     </row>
     <row r="73" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B73" s="6"/>
-      <c r="C73" s="41" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="D73" s="9" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
+      <c r="C73" s="41"/>
+      <c r="D73" s="9"/>
       <c r="E73" s="9"/>
       <c r="F73" s="9"/>
       <c r="G73" s="10"/>
       <c r="I73" s="6"/>
-      <c r="J73" s="28" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K73" s="3" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L73" s="3" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M73" s="3" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N73" s="29" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J73" s="28"/>
+      <c r="K73" s="3"/>
+      <c r="L73" s="3"/>
+      <c r="M73" s="3"/>
+      <c r="N73" s="29"/>
       <c r="P73" s="6"/>
       <c r="Q73" s="8"/>
       <c r="R73" s="8"/>
@@ -22080,38 +21153,17 @@
     </row>
     <row r="74" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B74" s="6"/>
-      <c r="C74" s="41" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="D74" s="9" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
+      <c r="C74" s="41"/>
+      <c r="D74" s="9"/>
       <c r="E74" s="9"/>
       <c r="F74" s="9"/>
       <c r="G74" s="10"/>
       <c r="I74" s="6"/>
-      <c r="J74" s="28" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K74" s="3" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L74" s="3" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M74" s="3" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N74" s="29" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J74" s="28"/>
+      <c r="K74" s="3"/>
+      <c r="L74" s="3"/>
+      <c r="M74" s="3"/>
+      <c r="N74" s="29"/>
       <c r="P74" s="6"/>
       <c r="Q74" s="8"/>
       <c r="R74" s="8"/>
@@ -22128,38 +21180,17 @@
     </row>
     <row r="75" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B75" s="6"/>
-      <c r="C75" s="41" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="D75" s="9" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
+      <c r="C75" s="41"/>
+      <c r="D75" s="9"/>
       <c r="E75" s="9"/>
       <c r="F75" s="9"/>
       <c r="G75" s="10"/>
       <c r="I75" s="6"/>
-      <c r="J75" s="28" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K75" s="3" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L75" s="3" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M75" s="3" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N75" s="29" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J75" s="28"/>
+      <c r="K75" s="3"/>
+      <c r="L75" s="3"/>
+      <c r="M75" s="3"/>
+      <c r="N75" s="29"/>
       <c r="P75" s="6"/>
       <c r="Q75" s="8"/>
       <c r="R75" s="8"/>
@@ -22176,38 +21207,17 @@
     </row>
     <row r="76" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B76" s="6"/>
-      <c r="C76" s="41" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="D76" s="9" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
+      <c r="C76" s="41"/>
+      <c r="D76" s="9"/>
       <c r="E76" s="9"/>
       <c r="F76" s="9"/>
       <c r="G76" s="10"/>
       <c r="I76" s="6"/>
-      <c r="J76" s="28" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K76" s="3" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L76" s="3" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M76" s="3" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N76" s="29" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J76" s="28"/>
+      <c r="K76" s="3"/>
+      <c r="L76" s="3"/>
+      <c r="M76" s="3"/>
+      <c r="N76" s="29"/>
       <c r="P76" s="6"/>
       <c r="Q76" s="8"/>
       <c r="R76" s="8"/>
@@ -22224,38 +21234,17 @@
     </row>
     <row r="77" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B77" s="6"/>
-      <c r="C77" s="41" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="D77" s="9" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
+      <c r="C77" s="41"/>
+      <c r="D77" s="9"/>
       <c r="E77" s="9"/>
       <c r="F77" s="9"/>
       <c r="G77" s="10"/>
       <c r="I77" s="6"/>
-      <c r="J77" s="28" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K77" s="3" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L77" s="3" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M77" s="3" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N77" s="29" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J77" s="28"/>
+      <c r="K77" s="3"/>
+      <c r="L77" s="3"/>
+      <c r="M77" s="3"/>
+      <c r="N77" s="29"/>
       <c r="P77" s="6"/>
       <c r="Q77" s="8"/>
       <c r="R77" s="8"/>
@@ -22347,213 +21336,87 @@
     </row>
     <row r="84" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B84" s="6"/>
-      <c r="C84" s="41" t="str">
-        <f>IF(SUM($E84:$G84)=0,"",SUM($E84:$G84))</f>
-        <v/>
-      </c>
-      <c r="D84" s="9" t="str">
-        <f>IF(SUM($E84:$F84)=0,"",SUM($E84:$F84))</f>
-        <v/>
-      </c>
+      <c r="C84" s="41"/>
+      <c r="D84" s="9"/>
       <c r="E84" s="9"/>
       <c r="F84" s="9"/>
       <c r="G84" s="10"/>
       <c r="I84" s="6"/>
-      <c r="J84" s="28" t="e">
-        <f>IFERROR((C84-C$84)/C$84,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K84" s="3" t="e">
-        <f t="shared" ref="K84" si="25">IFERROR((D84-D$84)/D$84,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="L84" s="3" t="e">
-        <f>IF(E84="",NA(),IFERROR((E84-E$84)/E$84,NA()))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="M84" s="3" t="e">
-        <f t="shared" ref="M84:N84" si="26">IF(F84="",NA(),IFERROR((F84-F$84)/F$84,NA()))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="N84" s="29" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J84" s="28"/>
+      <c r="K84" s="3"/>
+      <c r="L84" s="3"/>
+      <c r="M84" s="3"/>
+      <c r="N84" s="29"/>
     </row>
     <row r="85" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B85" s="6"/>
-      <c r="C85" s="41" t="str">
-        <f t="shared" ref="C85:C96" si="27">IF(SUM($E85:$G85)=0,"",SUM($E85:$G85))</f>
-        <v/>
-      </c>
-      <c r="D85" s="9" t="str">
-        <f t="shared" ref="D85:D96" si="28">IF(SUM($E85:$F85)=0,"",SUM($E85:$F85))</f>
-        <v/>
-      </c>
+      <c r="C85" s="41"/>
+      <c r="D85" s="9"/>
       <c r="E85" s="9"/>
       <c r="F85" s="9"/>
       <c r="G85" s="10"/>
       <c r="I85" s="6"/>
-      <c r="J85" s="28" t="e">
-        <f>IFERROR((C85-C$84)/C$84,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K85" s="3" t="e">
-        <f t="shared" ref="K85" si="29">IFERROR((D85-D$84)/D$84,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="L85" s="3" t="e">
-        <f t="shared" ref="L85:L96" si="30">IF(E85="",NA(),IFERROR((E85-E$84)/E$84,NA()))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="M85" s="3" t="e">
-        <f t="shared" ref="M85:M96" si="31">IF(F85="",NA(),IFERROR((F85-F$84)/F$84,NA()))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="N85" s="29" t="e">
-        <f t="shared" ref="N85:N96" si="32">IF(G85="",NA(),IFERROR((G85-G$84)/G$84,NA()))</f>
-        <v>#N/A</v>
-      </c>
+      <c r="J85" s="28"/>
+      <c r="K85" s="3"/>
+      <c r="L85" s="3"/>
+      <c r="M85" s="3"/>
+      <c r="N85" s="29"/>
     </row>
     <row r="86" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B86" s="6"/>
-      <c r="C86" s="41" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="D86" s="9" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
+      <c r="C86" s="41"/>
+      <c r="D86" s="9"/>
       <c r="E86" s="9"/>
       <c r="F86" s="9"/>
       <c r="G86" s="10"/>
       <c r="I86" s="6"/>
-      <c r="J86" s="28" t="e">
-        <f t="shared" ref="J86:J96" si="33">IFERROR((C86-C$84)/C$84,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K86" s="3" t="e">
-        <f t="shared" ref="K86:K96" si="34">IFERROR((D86-D$84)/D$84,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="L86" s="3" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M86" s="3" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N86" s="29" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J86" s="28"/>
+      <c r="K86" s="3"/>
+      <c r="L86" s="3"/>
+      <c r="M86" s="3"/>
+      <c r="N86" s="29"/>
     </row>
     <row r="87" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B87" s="6"/>
-      <c r="C87" s="41" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="D87" s="9" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
+      <c r="C87" s="41"/>
+      <c r="D87" s="9"/>
       <c r="E87" s="9"/>
       <c r="F87" s="9"/>
       <c r="G87" s="10"/>
       <c r="I87" s="6"/>
-      <c r="J87" s="28" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K87" s="3" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L87" s="3" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M87" s="3" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N87" s="29" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J87" s="28"/>
+      <c r="K87" s="3"/>
+      <c r="L87" s="3"/>
+      <c r="M87" s="3"/>
+      <c r="N87" s="29"/>
     </row>
     <row r="88" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B88" s="6"/>
-      <c r="C88" s="41" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="D88" s="9" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
+      <c r="C88" s="41"/>
+      <c r="D88" s="9"/>
       <c r="E88" s="9"/>
       <c r="F88" s="9"/>
       <c r="G88" s="10"/>
       <c r="I88" s="6"/>
-      <c r="J88" s="28" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K88" s="3" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L88" s="3" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M88" s="3" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N88" s="29" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J88" s="28"/>
+      <c r="K88" s="3"/>
+      <c r="L88" s="3"/>
+      <c r="M88" s="3"/>
+      <c r="N88" s="29"/>
     </row>
     <row r="89" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B89" s="6"/>
-      <c r="C89" s="41" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="D89" s="9" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
+      <c r="C89" s="41"/>
+      <c r="D89" s="9"/>
       <c r="E89" s="9"/>
       <c r="F89" s="9"/>
       <c r="G89" s="10"/>
       <c r="I89" s="6"/>
-      <c r="J89" s="28" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K89" s="3" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L89" s="3" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M89" s="3" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N89" s="29" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J89" s="28"/>
+      <c r="K89" s="3"/>
+      <c r="L89" s="3"/>
+      <c r="M89" s="3"/>
+      <c r="N89" s="29"/>
       <c r="P89" s="6"/>
       <c r="Q89" s="8"/>
       <c r="R89" s="8"/>
@@ -22570,38 +21433,17 @@
     </row>
     <row r="90" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B90" s="6"/>
-      <c r="C90" s="41" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="D90" s="9" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
+      <c r="C90" s="41"/>
+      <c r="D90" s="9"/>
       <c r="E90" s="9"/>
       <c r="F90" s="9"/>
       <c r="G90" s="10"/>
       <c r="I90" s="6"/>
-      <c r="J90" s="28" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K90" s="3" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L90" s="3" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M90" s="3" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N90" s="29" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J90" s="28"/>
+      <c r="K90" s="3"/>
+      <c r="L90" s="3"/>
+      <c r="M90" s="3"/>
+      <c r="N90" s="29"/>
       <c r="P90" s="6"/>
       <c r="Q90" s="8"/>
       <c r="R90" s="8"/>
@@ -22618,38 +21460,17 @@
     </row>
     <row r="91" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B91" s="6"/>
-      <c r="C91" s="41" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="D91" s="9" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
+      <c r="C91" s="41"/>
+      <c r="D91" s="9"/>
       <c r="E91" s="9"/>
       <c r="F91" s="9"/>
       <c r="G91" s="10"/>
       <c r="I91" s="6"/>
-      <c r="J91" s="28" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K91" s="3" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L91" s="3" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M91" s="3" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N91" s="29" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J91" s="28"/>
+      <c r="K91" s="3"/>
+      <c r="L91" s="3"/>
+      <c r="M91" s="3"/>
+      <c r="N91" s="29"/>
       <c r="P91" s="6"/>
       <c r="Q91" s="8"/>
       <c r="R91" s="8"/>
@@ -22666,38 +21487,17 @@
     </row>
     <row r="92" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B92" s="6"/>
-      <c r="C92" s="41" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="D92" s="9" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
+      <c r="C92" s="41"/>
+      <c r="D92" s="9"/>
       <c r="E92" s="9"/>
       <c r="F92" s="9"/>
       <c r="G92" s="10"/>
       <c r="I92" s="6"/>
-      <c r="J92" s="28" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K92" s="3" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L92" s="3" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M92" s="3" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N92" s="29" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J92" s="28"/>
+      <c r="K92" s="3"/>
+      <c r="L92" s="3"/>
+      <c r="M92" s="3"/>
+      <c r="N92" s="29"/>
       <c r="P92" s="6"/>
       <c r="Q92" s="8"/>
       <c r="R92" s="8"/>
@@ -22714,38 +21514,17 @@
     </row>
     <row r="93" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B93" s="6"/>
-      <c r="C93" s="41" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="D93" s="9" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
+      <c r="C93" s="41"/>
+      <c r="D93" s="9"/>
       <c r="E93" s="9"/>
       <c r="F93" s="9"/>
       <c r="G93" s="10"/>
       <c r="I93" s="6"/>
-      <c r="J93" s="28" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K93" s="3" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L93" s="3" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M93" s="3" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N93" s="29" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J93" s="28"/>
+      <c r="K93" s="3"/>
+      <c r="L93" s="3"/>
+      <c r="M93" s="3"/>
+      <c r="N93" s="29"/>
       <c r="P93" s="6"/>
       <c r="Q93" s="8"/>
       <c r="R93" s="8"/>
@@ -22762,38 +21541,17 @@
     </row>
     <row r="94" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B94" s="6"/>
-      <c r="C94" s="41" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="D94" s="9" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
+      <c r="C94" s="41"/>
+      <c r="D94" s="9"/>
       <c r="E94" s="9"/>
       <c r="F94" s="9"/>
       <c r="G94" s="10"/>
       <c r="I94" s="6"/>
-      <c r="J94" s="28" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K94" s="3" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L94" s="3" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M94" s="3" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N94" s="29" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J94" s="28"/>
+      <c r="K94" s="3"/>
+      <c r="L94" s="3"/>
+      <c r="M94" s="3"/>
+      <c r="N94" s="29"/>
       <c r="P94" s="6"/>
       <c r="Q94" s="8"/>
       <c r="R94" s="8"/>
@@ -22810,38 +21568,17 @@
     </row>
     <row r="95" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B95" s="6"/>
-      <c r="C95" s="41" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="D95" s="9" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
+      <c r="C95" s="41"/>
+      <c r="D95" s="9"/>
       <c r="E95" s="9"/>
       <c r="F95" s="9"/>
       <c r="G95" s="10"/>
       <c r="I95" s="6"/>
-      <c r="J95" s="28" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K95" s="3" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L95" s="3" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M95" s="3" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N95" s="29" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J95" s="28"/>
+      <c r="K95" s="3"/>
+      <c r="L95" s="3"/>
+      <c r="M95" s="3"/>
+      <c r="N95" s="29"/>
       <c r="P95" s="6"/>
       <c r="Q95" s="8"/>
       <c r="R95" s="8"/>
@@ -22858,38 +21595,17 @@
     </row>
     <row r="96" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B96" s="6"/>
-      <c r="C96" s="41" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="D96" s="9" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
+      <c r="C96" s="41"/>
+      <c r="D96" s="9"/>
       <c r="E96" s="9"/>
       <c r="F96" s="9"/>
       <c r="G96" s="10"/>
       <c r="I96" s="6"/>
-      <c r="J96" s="28" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
-      </c>
-      <c r="K96" s="3" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L96" s="3" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M96" s="3" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N96" s="29" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
+      <c r="J96" s="28"/>
+      <c r="K96" s="3"/>
+      <c r="L96" s="3"/>
+      <c r="M96" s="3"/>
+      <c r="N96" s="29"/>
       <c r="P96" s="6"/>
       <c r="Q96" s="8"/>
       <c r="R96" s="8"/>
@@ -23221,16 +21937,6 @@
       <c r="AL116" s="8"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J65:N77">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>ISNA(J65)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J84:N96">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>ISNA(J84)</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
   <drawing r:id="rId1"/>
@@ -24548,6 +23254,7 @@
       </c>
     </row>
     <row r="105" spans="2:19" ht="45" x14ac:dyDescent="0.2">
+      <c r="C105" s="62"/>
       <c r="D105" s="20" t="s">
         <v>5</v>
       </c>
@@ -24573,1106 +23280,551 @@
         <f>IF(C64="","",C64)</f>
         <v/>
       </c>
-      <c r="D106" s="25" t="str">
-        <f>IF(D64="","",IF(D23="","-",(D64-D23)/D23))</f>
+      <c r="D106" s="25"/>
+      <c r="E106" s="26"/>
+      <c r="F106" s="26"/>
+      <c r="G106" s="26"/>
+      <c r="H106" s="26"/>
+    </row>
+    <row r="107" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B107" s="1" t="str">
+        <f t="shared" ref="B107:C107" si="0">IF(B65="","",B65)</f>
         <v/>
       </c>
-      <c r="E106" s="26" t="str">
-        <f t="shared" ref="E106:H106" si="0">IF(E64="","",IF(E23="","-",(E64-E23)/E23))</f>
-        <v/>
-      </c>
-      <c r="F106" s="26" t="str">
+      <c r="C107" s="6" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G106" s="26" t="str">
-        <f t="shared" si="0"/>
+      <c r="D107" s="28"/>
+      <c r="E107" s="12"/>
+      <c r="F107" s="12"/>
+      <c r="G107" s="12"/>
+      <c r="H107" s="12"/>
+    </row>
+    <row r="108" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B108" s="1" t="str">
+        <f t="shared" ref="B108:C108" si="1">IF(B66="","",B66)</f>
         <v/>
       </c>
-      <c r="H106" s="26" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="107" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B107" s="1" t="str">
-        <f t="shared" ref="B107:C107" si="1">IF(B65="","",B65)</f>
-        <v/>
-      </c>
-      <c r="C107" s="6" t="str">
+      <c r="C108" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="D107" s="28" t="str">
-        <f t="shared" ref="D107:H107" si="2">IF(D65="","",IF(D24="","-",(D65-D24)/D24))</f>
+      <c r="D108" s="28"/>
+      <c r="E108" s="12"/>
+      <c r="F108" s="12"/>
+      <c r="G108" s="12"/>
+      <c r="H108" s="12"/>
+    </row>
+    <row r="109" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B109" s="1" t="str">
+        <f t="shared" ref="B109:C109" si="2">IF(B67="","",B67)</f>
         <v/>
       </c>
-      <c r="E107" s="12" t="str">
+      <c r="C109" s="6" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="F107" s="12" t="str">
-        <f t="shared" si="2"/>
+      <c r="D109" s="28"/>
+      <c r="E109" s="12"/>
+      <c r="F109" s="12"/>
+      <c r="G109" s="12"/>
+      <c r="H109" s="12"/>
+    </row>
+    <row r="110" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B110" s="1" t="str">
+        <f t="shared" ref="B110:C110" si="3">IF(B68="","",B68)</f>
         <v/>
       </c>
-      <c r="G107" s="12" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="H107" s="12" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="108" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B108" s="1" t="str">
-        <f t="shared" ref="B108:C108" si="3">IF(B66="","",B66)</f>
-        <v/>
-      </c>
-      <c r="C108" s="6" t="str">
+      <c r="C110" s="6" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="D108" s="28" t="str">
-        <f t="shared" ref="D108:H108" si="4">IF(D66="","",IF(D25="","-",(D66-D25)/D25))</f>
+      <c r="D110" s="28"/>
+      <c r="E110" s="12"/>
+      <c r="F110" s="12"/>
+      <c r="G110" s="12"/>
+      <c r="H110" s="12"/>
+    </row>
+    <row r="111" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B111" s="1" t="str">
+        <f t="shared" ref="B111:C111" si="4">IF(B69="","",B69)</f>
         <v/>
       </c>
-      <c r="E108" s="12" t="str">
+      <c r="C111" s="6" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="F108" s="12" t="str">
-        <f t="shared" si="4"/>
+      <c r="D111" s="28"/>
+      <c r="E111" s="12"/>
+      <c r="F111" s="12"/>
+      <c r="G111" s="12"/>
+      <c r="H111" s="12"/>
+    </row>
+    <row r="112" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="B112" s="1" t="str">
+        <f t="shared" ref="B112:C112" si="5">IF(B70="","",B70)</f>
         <v/>
       </c>
-      <c r="G108" s="12" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H108" s="12" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="109" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B109" s="1" t="str">
-        <f t="shared" ref="B109:C109" si="5">IF(B67="","",B67)</f>
-        <v/>
-      </c>
-      <c r="C109" s="6" t="str">
+      <c r="C112" s="6" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="D109" s="28" t="str">
-        <f t="shared" ref="D109:H109" si="6">IF(D67="","",IF(D26="","-",(D67-D26)/D26))</f>
+      <c r="D112" s="28"/>
+      <c r="E112" s="12"/>
+      <c r="F112" s="12"/>
+      <c r="G112" s="12"/>
+      <c r="H112" s="12"/>
+    </row>
+    <row r="113" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B113" s="1" t="str">
+        <f t="shared" ref="B113:C113" si="6">IF(B71="","",B71)</f>
         <v/>
       </c>
-      <c r="E109" s="12" t="str">
+      <c r="C113" s="6" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="F109" s="12" t="str">
-        <f t="shared" si="6"/>
+      <c r="D113" s="28"/>
+      <c r="E113" s="12"/>
+      <c r="F113" s="12"/>
+      <c r="G113" s="12"/>
+      <c r="H113" s="12"/>
+    </row>
+    <row r="114" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B114" s="1" t="str">
+        <f t="shared" ref="B114:C114" si="7">IF(B72="","",B72)</f>
         <v/>
       </c>
-      <c r="G109" s="12" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H109" s="12" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-    </row>
-    <row r="110" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B110" s="1" t="str">
-        <f t="shared" ref="B110:C110" si="7">IF(B68="","",B68)</f>
-        <v/>
-      </c>
-      <c r="C110" s="6" t="str">
+      <c r="C114" s="6" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="D110" s="28" t="str">
-        <f t="shared" ref="D110:H110" si="8">IF(D68="","",IF(D27="","-",(D68-D27)/D27))</f>
+      <c r="D114" s="28"/>
+      <c r="E114" s="12"/>
+      <c r="F114" s="12"/>
+      <c r="G114" s="12"/>
+      <c r="H114" s="12"/>
+    </row>
+    <row r="115" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B115" s="1" t="str">
+        <f t="shared" ref="B115:C115" si="8">IF(B73="","",B73)</f>
         <v/>
       </c>
-      <c r="E110" s="12" t="str">
+      <c r="C115" s="6" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="F110" s="12" t="str">
-        <f t="shared" si="8"/>
+      <c r="D115" s="28"/>
+      <c r="E115" s="12"/>
+      <c r="F115" s="12"/>
+      <c r="G115" s="12"/>
+      <c r="H115" s="12"/>
+    </row>
+    <row r="116" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B116" s="1" t="str">
+        <f t="shared" ref="B116:C116" si="9">IF(B74="","",B74)</f>
         <v/>
       </c>
-      <c r="G110" s="12" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H110" s="12" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-    </row>
-    <row r="111" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B111" s="1" t="str">
-        <f t="shared" ref="B111:C111" si="9">IF(B69="","",B69)</f>
-        <v/>
-      </c>
-      <c r="C111" s="6" t="str">
+      <c r="C116" s="6" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="D111" s="28" t="str">
-        <f t="shared" ref="D111:H111" si="10">IF(D69="","",IF(D28="","-",(D69-D28)/D28))</f>
+      <c r="D116" s="28"/>
+      <c r="E116" s="12"/>
+      <c r="F116" s="12"/>
+      <c r="G116" s="12"/>
+      <c r="H116" s="12"/>
+    </row>
+    <row r="117" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B117" s="1" t="str">
+        <f t="shared" ref="B117:C117" si="10">IF(B75="","",B75)</f>
         <v/>
       </c>
-      <c r="E111" s="12" t="str">
+      <c r="C117" s="6" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="F111" s="12" t="str">
-        <f t="shared" si="10"/>
+      <c r="D117" s="28"/>
+      <c r="E117" s="12"/>
+      <c r="F117" s="12"/>
+      <c r="G117" s="12"/>
+      <c r="H117" s="12"/>
+    </row>
+    <row r="118" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B118" s="1" t="str">
+        <f t="shared" ref="B118:C118" si="11">IF(B76="","",B76)</f>
         <v/>
       </c>
-      <c r="G111" s="12" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="H111" s="12" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-    </row>
-    <row r="112" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B112" s="1" t="str">
-        <f t="shared" ref="B112:C112" si="11">IF(B70="","",B70)</f>
-        <v/>
-      </c>
-      <c r="C112" s="6" t="str">
+      <c r="C118" s="6" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="D112" s="28" t="str">
-        <f t="shared" ref="D112:H112" si="12">IF(D70="","",IF(D29="","-",(D70-D29)/D29))</f>
+      <c r="D118" s="28"/>
+      <c r="E118" s="12"/>
+      <c r="F118" s="12"/>
+      <c r="G118" s="12"/>
+      <c r="H118" s="12"/>
+    </row>
+    <row r="119" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B119" s="1" t="str">
+        <f t="shared" ref="B119:C119" si="12">IF(B77="","",B77)</f>
         <v/>
       </c>
-      <c r="E112" s="12" t="str">
+      <c r="C119" s="6" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
-      <c r="F112" s="12" t="str">
-        <f t="shared" si="12"/>
+      <c r="D119" s="28"/>
+      <c r="E119" s="12"/>
+      <c r="F119" s="12"/>
+      <c r="G119" s="12"/>
+      <c r="H119" s="12"/>
+    </row>
+    <row r="120" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B120" s="1" t="str">
+        <f t="shared" ref="B120:C120" si="13">IF(B78="","",B78)</f>
         <v/>
       </c>
-      <c r="G112" s="12" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="H112" s="12" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-    </row>
-    <row r="113" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B113" s="1" t="str">
-        <f t="shared" ref="B113:C113" si="13">IF(B71="","",B71)</f>
-        <v/>
-      </c>
-      <c r="C113" s="6" t="str">
+      <c r="C120" s="6" t="str">
         <f t="shared" si="13"/>
         <v/>
       </c>
-      <c r="D113" s="28" t="str">
-        <f t="shared" ref="D113:H113" si="14">IF(D71="","",IF(D30="","-",(D71-D30)/D30))</f>
+      <c r="D120" s="28"/>
+      <c r="E120" s="12"/>
+      <c r="F120" s="12"/>
+      <c r="G120" s="12"/>
+      <c r="H120" s="12"/>
+    </row>
+    <row r="121" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B121" s="1" t="str">
+        <f t="shared" ref="B121:C121" si="14">IF(B79="","",B79)</f>
         <v/>
       </c>
-      <c r="E113" s="12" t="str">
+      <c r="C121" s="6" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="F113" s="12" t="str">
-        <f t="shared" si="14"/>
+      <c r="D121" s="28"/>
+      <c r="E121" s="12"/>
+      <c r="F121" s="12"/>
+      <c r="G121" s="12"/>
+      <c r="H121" s="12"/>
+    </row>
+    <row r="122" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B122" s="1" t="str">
+        <f t="shared" ref="B122:C122" si="15">IF(B80="","",B80)</f>
         <v/>
       </c>
-      <c r="G113" s="12" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="H113" s="12" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-    </row>
-    <row r="114" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B114" s="1" t="str">
-        <f t="shared" ref="B114:C114" si="15">IF(B72="","",B72)</f>
-        <v/>
-      </c>
-      <c r="C114" s="6" t="str">
+      <c r="C122" s="6" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="D114" s="28" t="str">
-        <f t="shared" ref="D114:H114" si="16">IF(D72="","",IF(D31="","-",(D72-D31)/D31))</f>
+      <c r="D122" s="28"/>
+      <c r="E122" s="12"/>
+      <c r="F122" s="12"/>
+      <c r="G122" s="12"/>
+      <c r="H122" s="12"/>
+    </row>
+    <row r="123" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B123" s="1" t="str">
+        <f t="shared" ref="B123:C123" si="16">IF(B81="","",B81)</f>
         <v/>
       </c>
-      <c r="E114" s="12" t="str">
+      <c r="C123" s="6" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
-      <c r="F114" s="12" t="str">
-        <f t="shared" si="16"/>
+      <c r="D123" s="28"/>
+      <c r="E123" s="12"/>
+      <c r="F123" s="12"/>
+      <c r="G123" s="12"/>
+      <c r="H123" s="12"/>
+    </row>
+    <row r="124" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B124" s="1" t="str">
+        <f t="shared" ref="B124:C124" si="17">IF(B82="","",B82)</f>
         <v/>
       </c>
-      <c r="G114" s="12" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="H114" s="12" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-    </row>
-    <row r="115" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B115" s="1" t="str">
-        <f t="shared" ref="B115:C115" si="17">IF(B73="","",B73)</f>
-        <v/>
-      </c>
-      <c r="C115" s="6" t="str">
+      <c r="C124" s="6" t="str">
         <f t="shared" si="17"/>
         <v/>
       </c>
-      <c r="D115" s="28" t="str">
-        <f t="shared" ref="D115:H115" si="18">IF(D73="","",IF(D32="","-",(D73-D32)/D32))</f>
+      <c r="D124" s="28"/>
+      <c r="E124" s="12"/>
+      <c r="F124" s="12"/>
+      <c r="G124" s="12"/>
+      <c r="H124" s="12"/>
+    </row>
+    <row r="125" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B125" s="1" t="str">
+        <f t="shared" ref="B125:C125" si="18">IF(B83="","",B83)</f>
         <v/>
       </c>
-      <c r="E115" s="12" t="str">
+      <c r="C125" s="6" t="str">
         <f t="shared" si="18"/>
         <v/>
       </c>
-      <c r="F115" s="12" t="str">
-        <f t="shared" si="18"/>
+      <c r="D125" s="28"/>
+      <c r="E125" s="12"/>
+      <c r="F125" s="12"/>
+      <c r="G125" s="12"/>
+      <c r="H125" s="12"/>
+    </row>
+    <row r="126" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B126" s="1" t="str">
+        <f t="shared" ref="B126:C126" si="19">IF(B84="","",B84)</f>
         <v/>
       </c>
-      <c r="G115" s="12" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="H115" s="12" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-    </row>
-    <row r="116" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B116" s="1" t="str">
-        <f t="shared" ref="B116:C116" si="19">IF(B74="","",B74)</f>
-        <v/>
-      </c>
-      <c r="C116" s="6" t="str">
+      <c r="C126" s="6" t="str">
         <f t="shared" si="19"/>
         <v/>
       </c>
-      <c r="D116" s="28" t="str">
-        <f t="shared" ref="D116:H116" si="20">IF(D74="","",IF(D33="","-",(D74-D33)/D33))</f>
+      <c r="D126" s="28"/>
+      <c r="E126" s="12"/>
+      <c r="F126" s="12"/>
+      <c r="G126" s="12"/>
+      <c r="H126" s="12"/>
+    </row>
+    <row r="127" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B127" s="1" t="str">
+        <f t="shared" ref="B127:C127" si="20">IF(B85="","",B85)</f>
         <v/>
       </c>
-      <c r="E116" s="12" t="str">
+      <c r="C127" s="6" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="F116" s="12" t="str">
-        <f t="shared" si="20"/>
+      <c r="D127" s="28"/>
+      <c r="E127" s="12"/>
+      <c r="F127" s="12"/>
+      <c r="G127" s="12"/>
+      <c r="H127" s="12"/>
+    </row>
+    <row r="128" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B128" s="1" t="str">
+        <f t="shared" ref="B128:C128" si="21">IF(B86="","",B86)</f>
         <v/>
       </c>
-      <c r="G116" s="12" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="H116" s="12" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-    </row>
-    <row r="117" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B117" s="1" t="str">
-        <f t="shared" ref="B117:C117" si="21">IF(B75="","",B75)</f>
-        <v/>
-      </c>
-      <c r="C117" s="6" t="str">
+      <c r="C128" s="6" t="str">
         <f t="shared" si="21"/>
         <v/>
       </c>
-      <c r="D117" s="28" t="str">
-        <f t="shared" ref="D117:H117" si="22">IF(D75="","",IF(D34="","-",(D75-D34)/D34))</f>
+      <c r="D128" s="28"/>
+      <c r="E128" s="12"/>
+      <c r="F128" s="12"/>
+      <c r="G128" s="12"/>
+      <c r="H128" s="12"/>
+    </row>
+    <row r="129" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B129" s="1" t="str">
+        <f t="shared" ref="B129:C129" si="22">IF(B87="","",B87)</f>
         <v/>
       </c>
-      <c r="E117" s="12" t="str">
+      <c r="C129" s="6" t="str">
         <f t="shared" si="22"/>
         <v/>
       </c>
-      <c r="F117" s="12" t="str">
-        <f t="shared" si="22"/>
+      <c r="D129" s="28"/>
+      <c r="E129" s="12"/>
+      <c r="F129" s="12"/>
+      <c r="G129" s="12"/>
+      <c r="H129" s="12"/>
+    </row>
+    <row r="130" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B130" s="1" t="str">
+        <f t="shared" ref="B130:C130" si="23">IF(B88="","",B88)</f>
         <v/>
       </c>
-      <c r="G117" s="12" t="str">
-        <f t="shared" si="22"/>
-        <v/>
-      </c>
-      <c r="H117" s="12" t="str">
-        <f t="shared" si="22"/>
-        <v/>
-      </c>
-    </row>
-    <row r="118" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B118" s="1" t="str">
-        <f t="shared" ref="B118:C118" si="23">IF(B76="","",B76)</f>
-        <v/>
-      </c>
-      <c r="C118" s="6" t="str">
+      <c r="C130" s="6" t="str">
         <f t="shared" si="23"/>
         <v/>
       </c>
-      <c r="D118" s="28" t="str">
-        <f t="shared" ref="D118:H118" si="24">IF(D76="","",IF(D35="","-",(D76-D35)/D35))</f>
+      <c r="D130" s="28"/>
+      <c r="E130" s="12"/>
+      <c r="F130" s="12"/>
+      <c r="G130" s="12"/>
+      <c r="H130" s="12"/>
+    </row>
+    <row r="131" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B131" s="1" t="str">
+        <f t="shared" ref="B131:C131" si="24">IF(B89="","",B89)</f>
         <v/>
       </c>
-      <c r="E118" s="12" t="str">
+      <c r="C131" s="6" t="str">
         <f t="shared" si="24"/>
         <v/>
       </c>
-      <c r="F118" s="12" t="str">
-        <f t="shared" si="24"/>
+      <c r="D131" s="44"/>
+      <c r="E131" s="45"/>
+      <c r="F131" s="45"/>
+      <c r="G131" s="45"/>
+      <c r="H131" s="45"/>
+    </row>
+    <row r="132" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B132" s="1" t="str">
+        <f t="shared" ref="B132:C132" si="25">IF(B90="","",B90)</f>
         <v/>
       </c>
-      <c r="G118" s="12" t="str">
-        <f t="shared" si="24"/>
-        <v/>
-      </c>
-      <c r="H118" s="12" t="str">
-        <f t="shared" si="24"/>
-        <v/>
-      </c>
-    </row>
-    <row r="119" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B119" s="1" t="str">
-        <f t="shared" ref="B119:C119" si="25">IF(B77="","",B77)</f>
-        <v/>
-      </c>
-      <c r="C119" s="6" t="str">
+      <c r="C132" s="6" t="str">
         <f t="shared" si="25"/>
         <v/>
       </c>
-      <c r="D119" s="28" t="str">
-        <f t="shared" ref="D119:H119" si="26">IF(D77="","",IF(D36="","-",(D77-D36)/D36))</f>
+      <c r="D132" s="44"/>
+      <c r="E132" s="45"/>
+      <c r="F132" s="45"/>
+      <c r="G132" s="45"/>
+      <c r="H132" s="45"/>
+    </row>
+    <row r="133" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B133" s="1" t="str">
+        <f t="shared" ref="B133:C133" si="26">IF(B91="","",B91)</f>
         <v/>
       </c>
-      <c r="E119" s="12" t="str">
+      <c r="C133" s="6" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="F119" s="12" t="str">
-        <f t="shared" si="26"/>
+      <c r="D133" s="44"/>
+      <c r="E133" s="45"/>
+      <c r="F133" s="45"/>
+      <c r="G133" s="45"/>
+      <c r="H133" s="45"/>
+    </row>
+    <row r="134" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B134" s="1" t="str">
+        <f t="shared" ref="B134:C134" si="27">IF(B92="","",B92)</f>
         <v/>
       </c>
-      <c r="G119" s="12" t="str">
-        <f t="shared" si="26"/>
-        <v/>
-      </c>
-      <c r="H119" s="12" t="str">
-        <f t="shared" si="26"/>
-        <v/>
-      </c>
-    </row>
-    <row r="120" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B120" s="1" t="str">
-        <f t="shared" ref="B120:C120" si="27">IF(B78="","",B78)</f>
-        <v/>
-      </c>
-      <c r="C120" s="6" t="str">
+      <c r="C134" s="6" t="str">
         <f t="shared" si="27"/>
         <v/>
       </c>
-      <c r="D120" s="28" t="str">
-        <f t="shared" ref="D120:H120" si="28">IF(D78="","",IF(D37="","-",(D78-D37)/D37))</f>
+      <c r="D134" s="44"/>
+      <c r="E134" s="45"/>
+      <c r="F134" s="45"/>
+      <c r="G134" s="45"/>
+      <c r="H134" s="45"/>
+    </row>
+    <row r="135" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B135" s="1" t="str">
+        <f t="shared" ref="B135:C135" si="28">IF(B93="","",B93)</f>
         <v/>
       </c>
-      <c r="E120" s="12" t="str">
+      <c r="C135" s="6" t="str">
         <f t="shared" si="28"/>
         <v/>
       </c>
-      <c r="F120" s="12" t="str">
-        <f t="shared" si="28"/>
+      <c r="D135" s="44"/>
+      <c r="E135" s="45"/>
+      <c r="F135" s="45"/>
+      <c r="G135" s="45"/>
+      <c r="H135" s="45"/>
+    </row>
+    <row r="136" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B136" s="1" t="str">
+        <f t="shared" ref="B136:C136" si="29">IF(B94="","",B94)</f>
         <v/>
       </c>
-      <c r="G120" s="12" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
-      <c r="H120" s="12" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
-    </row>
-    <row r="121" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B121" s="1" t="str">
-        <f t="shared" ref="B121:C121" si="29">IF(B79="","",B79)</f>
-        <v/>
-      </c>
-      <c r="C121" s="6" t="str">
+      <c r="C136" s="6" t="str">
         <f t="shared" si="29"/>
         <v/>
       </c>
-      <c r="D121" s="28" t="str">
-        <f t="shared" ref="D121:H121" si="30">IF(D79="","",IF(D38="","-",(D79-D38)/D38))</f>
+      <c r="D136" s="44"/>
+      <c r="E136" s="45"/>
+      <c r="F136" s="45"/>
+      <c r="G136" s="45"/>
+      <c r="H136" s="45"/>
+    </row>
+    <row r="137" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B137" s="1" t="str">
+        <f t="shared" ref="B137:C137" si="30">IF(B95="","",B95)</f>
         <v/>
       </c>
-      <c r="E121" s="12" t="str">
+      <c r="C137" s="6" t="str">
         <f t="shared" si="30"/>
         <v/>
       </c>
-      <c r="F121" s="12" t="str">
-        <f t="shared" si="30"/>
+      <c r="D137" s="44"/>
+      <c r="E137" s="45"/>
+      <c r="F137" s="45"/>
+      <c r="G137" s="45"/>
+      <c r="H137" s="45"/>
+    </row>
+    <row r="138" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B138" s="1" t="str">
+        <f t="shared" ref="B138:C138" si="31">IF(B96="","",B96)</f>
         <v/>
       </c>
-      <c r="G121" s="12" t="str">
-        <f t="shared" si="30"/>
-        <v/>
-      </c>
-      <c r="H121" s="12" t="str">
-        <f t="shared" si="30"/>
-        <v/>
-      </c>
-    </row>
-    <row r="122" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B122" s="1" t="str">
-        <f t="shared" ref="B122:C122" si="31">IF(B80="","",B80)</f>
-        <v/>
-      </c>
-      <c r="C122" s="6" t="str">
+      <c r="C138" s="6" t="str">
         <f t="shared" si="31"/>
         <v/>
       </c>
-      <c r="D122" s="28" t="str">
-        <f t="shared" ref="D122:H122" si="32">IF(D80="","",IF(D39="","-",(D80-D39)/D39))</f>
+      <c r="D138" s="44"/>
+      <c r="E138" s="45"/>
+      <c r="F138" s="45"/>
+      <c r="G138" s="45"/>
+      <c r="H138" s="45"/>
+    </row>
+    <row r="139" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B139" s="1" t="str">
+        <f t="shared" ref="B139:C139" si="32">IF(B97="","",B97)</f>
         <v/>
       </c>
-      <c r="E122" s="12" t="str">
+      <c r="C139" s="6" t="str">
         <f t="shared" si="32"/>
         <v/>
       </c>
-      <c r="F122" s="12" t="str">
-        <f t="shared" si="32"/>
+      <c r="D139" s="44"/>
+      <c r="E139" s="45"/>
+      <c r="F139" s="45"/>
+      <c r="G139" s="45"/>
+      <c r="H139" s="45"/>
+    </row>
+    <row r="140" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B140" s="1" t="str">
+        <f t="shared" ref="B140:C140" si="33">IF(B98="","",B98)</f>
         <v/>
       </c>
-      <c r="G122" s="12" t="str">
-        <f t="shared" si="32"/>
-        <v/>
-      </c>
-      <c r="H122" s="12" t="str">
-        <f t="shared" si="32"/>
-        <v/>
-      </c>
-    </row>
-    <row r="123" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B123" s="1" t="str">
-        <f t="shared" ref="B123:C123" si="33">IF(B81="","",B81)</f>
-        <v/>
-      </c>
-      <c r="C123" s="6" t="str">
+      <c r="C140" s="6" t="str">
         <f t="shared" si="33"/>
         <v/>
       </c>
-      <c r="D123" s="28" t="str">
-        <f t="shared" ref="D123:H123" si="34">IF(D81="","",IF(D40="","-",(D81-D40)/D40))</f>
+      <c r="D140" s="44"/>
+      <c r="E140" s="45"/>
+      <c r="F140" s="45"/>
+      <c r="G140" s="45"/>
+      <c r="H140" s="45"/>
+    </row>
+    <row r="141" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B141" s="1" t="str">
+        <f t="shared" ref="B141:C141" si="34">IF(B99="","",B99)</f>
         <v/>
       </c>
-      <c r="E123" s="12" t="str">
+      <c r="C141" s="6" t="str">
         <f t="shared" si="34"/>
         <v/>
       </c>
-      <c r="F123" s="12" t="str">
-        <f t="shared" si="34"/>
+      <c r="D141" s="44"/>
+      <c r="E141" s="45"/>
+      <c r="F141" s="45"/>
+      <c r="G141" s="45"/>
+      <c r="H141" s="45"/>
+    </row>
+    <row r="142" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B142" s="1" t="str">
+        <f t="shared" ref="B142:C142" si="35">IF(B100="","",B100)</f>
         <v/>
       </c>
-      <c r="G123" s="12" t="str">
-        <f t="shared" si="34"/>
-        <v/>
-      </c>
-      <c r="H123" s="12" t="str">
-        <f t="shared" si="34"/>
-        <v/>
-      </c>
-    </row>
-    <row r="124" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B124" s="1" t="str">
-        <f t="shared" ref="B124:C124" si="35">IF(B82="","",B82)</f>
-        <v/>
-      </c>
-      <c r="C124" s="6" t="str">
+      <c r="C142" s="6" t="str">
         <f t="shared" si="35"/>
         <v/>
       </c>
-      <c r="D124" s="28" t="str">
-        <f t="shared" ref="D124:H124" si="36">IF(D82="","",IF(D41="","-",(D82-D41)/D41))</f>
-        <v/>
-      </c>
-      <c r="E124" s="12" t="str">
-        <f t="shared" si="36"/>
-        <v/>
-      </c>
-      <c r="F124" s="12" t="str">
-        <f t="shared" si="36"/>
-        <v/>
-      </c>
-      <c r="G124" s="12" t="str">
-        <f t="shared" si="36"/>
-        <v/>
-      </c>
-      <c r="H124" s="12" t="str">
-        <f t="shared" si="36"/>
-        <v/>
-      </c>
-    </row>
-    <row r="125" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B125" s="1" t="str">
-        <f t="shared" ref="B125:C125" si="37">IF(B83="","",B83)</f>
-        <v/>
-      </c>
-      <c r="C125" s="6" t="str">
-        <f t="shared" si="37"/>
-        <v/>
-      </c>
-      <c r="D125" s="28" t="str">
-        <f t="shared" ref="D125:H125" si="38">IF(D83="","",IF(D42="","-",(D83-D42)/D42))</f>
-        <v/>
-      </c>
-      <c r="E125" s="12" t="str">
-        <f t="shared" si="38"/>
-        <v/>
-      </c>
-      <c r="F125" s="12" t="str">
-        <f t="shared" si="38"/>
-        <v/>
-      </c>
-      <c r="G125" s="12" t="str">
-        <f t="shared" si="38"/>
-        <v/>
-      </c>
-      <c r="H125" s="12" t="str">
-        <f t="shared" si="38"/>
-        <v/>
-      </c>
-    </row>
-    <row r="126" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B126" s="1" t="str">
-        <f t="shared" ref="B126:C126" si="39">IF(B84="","",B84)</f>
-        <v/>
-      </c>
-      <c r="C126" s="6" t="str">
-        <f t="shared" si="39"/>
-        <v/>
-      </c>
-      <c r="D126" s="28" t="str">
-        <f t="shared" ref="D126:H126" si="40">IF(D84="","",IF(D43="","-",(D84-D43)/D43))</f>
-        <v/>
-      </c>
-      <c r="E126" s="12" t="str">
-        <f t="shared" si="40"/>
-        <v/>
-      </c>
-      <c r="F126" s="12" t="str">
-        <f t="shared" si="40"/>
-        <v/>
-      </c>
-      <c r="G126" s="12" t="str">
-        <f t="shared" si="40"/>
-        <v/>
-      </c>
-      <c r="H126" s="12" t="str">
-        <f t="shared" si="40"/>
-        <v/>
-      </c>
-    </row>
-    <row r="127" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B127" s="1" t="str">
-        <f t="shared" ref="B127:C127" si="41">IF(B85="","",B85)</f>
-        <v/>
-      </c>
-      <c r="C127" s="6" t="str">
-        <f t="shared" si="41"/>
-        <v/>
-      </c>
-      <c r="D127" s="28" t="str">
-        <f t="shared" ref="D127:H127" si="42">IF(D85="","",IF(D44="","-",(D85-D44)/D44))</f>
-        <v/>
-      </c>
-      <c r="E127" s="12" t="str">
-        <f t="shared" si="42"/>
-        <v/>
-      </c>
-      <c r="F127" s="12" t="str">
-        <f t="shared" si="42"/>
-        <v/>
-      </c>
-      <c r="G127" s="12" t="str">
-        <f t="shared" si="42"/>
-        <v/>
-      </c>
-      <c r="H127" s="12" t="str">
-        <f t="shared" si="42"/>
-        <v/>
-      </c>
-    </row>
-    <row r="128" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B128" s="1" t="str">
-        <f t="shared" ref="B128:C128" si="43">IF(B86="","",B86)</f>
-        <v/>
-      </c>
-      <c r="C128" s="6" t="str">
-        <f t="shared" si="43"/>
-        <v/>
-      </c>
-      <c r="D128" s="28" t="str">
-        <f t="shared" ref="D128:H128" si="44">IF(D86="","",IF(D45="","-",(D86-D45)/D45))</f>
-        <v/>
-      </c>
-      <c r="E128" s="12" t="str">
-        <f t="shared" si="44"/>
-        <v/>
-      </c>
-      <c r="F128" s="12" t="str">
-        <f t="shared" si="44"/>
-        <v/>
-      </c>
-      <c r="G128" s="12" t="str">
-        <f t="shared" si="44"/>
-        <v/>
-      </c>
-      <c r="H128" s="12" t="str">
-        <f t="shared" si="44"/>
-        <v/>
-      </c>
-    </row>
-    <row r="129" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B129" s="1" t="str">
-        <f t="shared" ref="B129:C129" si="45">IF(B87="","",B87)</f>
-        <v/>
-      </c>
-      <c r="C129" s="6" t="str">
-        <f t="shared" si="45"/>
-        <v/>
-      </c>
-      <c r="D129" s="28" t="str">
-        <f t="shared" ref="D129:H129" si="46">IF(D87="","",IF(D46="","-",(D87-D46)/D46))</f>
-        <v/>
-      </c>
-      <c r="E129" s="12" t="str">
-        <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="F129" s="12" t="str">
-        <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="G129" s="12" t="str">
-        <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="H129" s="12" t="str">
-        <f t="shared" si="46"/>
-        <v/>
-      </c>
-    </row>
-    <row r="130" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B130" s="1" t="str">
-        <f t="shared" ref="B130:C130" si="47">IF(B88="","",B88)</f>
-        <v/>
-      </c>
-      <c r="C130" s="6" t="str">
-        <f t="shared" si="47"/>
-        <v/>
-      </c>
-      <c r="D130" s="28" t="str">
-        <f t="shared" ref="D130:H130" si="48">IF(D88="","",IF(D47="","-",(D88-D47)/D47))</f>
-        <v/>
-      </c>
-      <c r="E130" s="12" t="str">
-        <f t="shared" si="48"/>
-        <v/>
-      </c>
-      <c r="F130" s="12" t="str">
-        <f t="shared" si="48"/>
-        <v/>
-      </c>
-      <c r="G130" s="12" t="str">
-        <f t="shared" si="48"/>
-        <v/>
-      </c>
-      <c r="H130" s="12" t="str">
-        <f t="shared" si="48"/>
-        <v/>
-      </c>
-    </row>
-    <row r="131" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B131" s="1" t="str">
-        <f t="shared" ref="B131:C131" si="49">IF(B89="","",B89)</f>
-        <v/>
-      </c>
-      <c r="C131" s="6" t="str">
-        <f t="shared" si="49"/>
-        <v/>
-      </c>
-      <c r="D131" s="44" t="str">
-        <f t="shared" ref="D131:H131" si="50">IF(D89="","",IF(D48="","-",(D89-D48)/D48))</f>
-        <v/>
-      </c>
-      <c r="E131" s="45" t="str">
-        <f t="shared" si="50"/>
-        <v/>
-      </c>
-      <c r="F131" s="45" t="str">
-        <f t="shared" si="50"/>
-        <v/>
-      </c>
-      <c r="G131" s="45" t="str">
-        <f t="shared" si="50"/>
-        <v/>
-      </c>
-      <c r="H131" s="45" t="str">
-        <f t="shared" si="50"/>
-        <v/>
-      </c>
-    </row>
-    <row r="132" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B132" s="1" t="str">
-        <f t="shared" ref="B132:C132" si="51">IF(B90="","",B90)</f>
-        <v/>
-      </c>
-      <c r="C132" s="6" t="str">
-        <f t="shared" si="51"/>
-        <v/>
-      </c>
-      <c r="D132" s="44" t="str">
-        <f t="shared" ref="D132:H132" si="52">IF(D90="","",IF(D49="","-",(D90-D49)/D49))</f>
-        <v/>
-      </c>
-      <c r="E132" s="45" t="str">
-        <f t="shared" si="52"/>
-        <v/>
-      </c>
-      <c r="F132" s="45" t="str">
-        <f t="shared" si="52"/>
-        <v/>
-      </c>
-      <c r="G132" s="45" t="str">
-        <f t="shared" si="52"/>
-        <v/>
-      </c>
-      <c r="H132" s="45" t="str">
-        <f t="shared" si="52"/>
-        <v/>
-      </c>
-    </row>
-    <row r="133" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B133" s="1" t="str">
-        <f t="shared" ref="B133:C133" si="53">IF(B91="","",B91)</f>
-        <v/>
-      </c>
-      <c r="C133" s="6" t="str">
-        <f t="shared" si="53"/>
-        <v/>
-      </c>
-      <c r="D133" s="44" t="str">
-        <f t="shared" ref="D133:H133" si="54">IF(D91="","",IF(D50="","-",(D91-D50)/D50))</f>
-        <v/>
-      </c>
-      <c r="E133" s="45" t="str">
-        <f t="shared" si="54"/>
-        <v/>
-      </c>
-      <c r="F133" s="45" t="str">
-        <f t="shared" si="54"/>
-        <v/>
-      </c>
-      <c r="G133" s="45" t="str">
-        <f t="shared" si="54"/>
-        <v/>
-      </c>
-      <c r="H133" s="45" t="str">
-        <f t="shared" si="54"/>
-        <v/>
-      </c>
-    </row>
-    <row r="134" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B134" s="1" t="str">
-        <f t="shared" ref="B134:C134" si="55">IF(B92="","",B92)</f>
-        <v/>
-      </c>
-      <c r="C134" s="6" t="str">
-        <f t="shared" si="55"/>
-        <v/>
-      </c>
-      <c r="D134" s="44" t="str">
-        <f t="shared" ref="D134:H134" si="56">IF(D92="","",IF(D51="","-",(D92-D51)/D51))</f>
-        <v/>
-      </c>
-      <c r="E134" s="45" t="str">
-        <f t="shared" si="56"/>
-        <v/>
-      </c>
-      <c r="F134" s="45" t="str">
-        <f t="shared" si="56"/>
-        <v/>
-      </c>
-      <c r="G134" s="45" t="str">
-        <f t="shared" si="56"/>
-        <v/>
-      </c>
-      <c r="H134" s="45" t="str">
-        <f t="shared" si="56"/>
-        <v/>
-      </c>
-    </row>
-    <row r="135" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B135" s="1" t="str">
-        <f t="shared" ref="B135:C135" si="57">IF(B93="","",B93)</f>
-        <v/>
-      </c>
-      <c r="C135" s="6" t="str">
-        <f t="shared" si="57"/>
-        <v/>
-      </c>
-      <c r="D135" s="44" t="str">
-        <f t="shared" ref="D135:H135" si="58">IF(D93="","",IF(D52="","-",(D93-D52)/D52))</f>
-        <v/>
-      </c>
-      <c r="E135" s="45" t="str">
-        <f t="shared" si="58"/>
-        <v/>
-      </c>
-      <c r="F135" s="45" t="str">
-        <f t="shared" si="58"/>
-        <v/>
-      </c>
-      <c r="G135" s="45" t="str">
-        <f t="shared" si="58"/>
-        <v/>
-      </c>
-      <c r="H135" s="45" t="str">
-        <f t="shared" si="58"/>
-        <v/>
-      </c>
-    </row>
-    <row r="136" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B136" s="1" t="str">
-        <f t="shared" ref="B136:C136" si="59">IF(B94="","",B94)</f>
-        <v/>
-      </c>
-      <c r="C136" s="6" t="str">
-        <f t="shared" si="59"/>
-        <v/>
-      </c>
-      <c r="D136" s="44" t="str">
-        <f t="shared" ref="D136:H136" si="60">IF(D94="","",IF(D53="","-",(D94-D53)/D53))</f>
-        <v/>
-      </c>
-      <c r="E136" s="45" t="str">
-        <f t="shared" si="60"/>
-        <v/>
-      </c>
-      <c r="F136" s="45" t="str">
-        <f t="shared" si="60"/>
-        <v/>
-      </c>
-      <c r="G136" s="45" t="str">
-        <f t="shared" si="60"/>
-        <v/>
-      </c>
-      <c r="H136" s="45" t="str">
-        <f t="shared" si="60"/>
-        <v/>
-      </c>
-    </row>
-    <row r="137" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B137" s="1" t="str">
-        <f t="shared" ref="B137:C137" si="61">IF(B95="","",B95)</f>
-        <v/>
-      </c>
-      <c r="C137" s="6" t="str">
-        <f t="shared" si="61"/>
-        <v/>
-      </c>
-      <c r="D137" s="44" t="str">
-        <f t="shared" ref="D137:H137" si="62">IF(D95="","",IF(D54="","-",(D95-D54)/D54))</f>
-        <v/>
-      </c>
-      <c r="E137" s="45" t="str">
-        <f t="shared" si="62"/>
-        <v/>
-      </c>
-      <c r="F137" s="45" t="str">
-        <f t="shared" si="62"/>
-        <v/>
-      </c>
-      <c r="G137" s="45" t="str">
-        <f t="shared" si="62"/>
-        <v/>
-      </c>
-      <c r="H137" s="45" t="str">
-        <f t="shared" si="62"/>
-        <v/>
-      </c>
-    </row>
-    <row r="138" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B138" s="1" t="str">
-        <f t="shared" ref="B138:C138" si="63">IF(B96="","",B96)</f>
-        <v/>
-      </c>
-      <c r="C138" s="6" t="str">
-        <f t="shared" si="63"/>
-        <v/>
-      </c>
-      <c r="D138" s="44" t="str">
-        <f t="shared" ref="D138:H138" si="64">IF(D96="","",IF(D55="","-",(D96-D55)/D55))</f>
-        <v/>
-      </c>
-      <c r="E138" s="45" t="str">
-        <f t="shared" si="64"/>
-        <v/>
-      </c>
-      <c r="F138" s="45" t="str">
-        <f t="shared" si="64"/>
-        <v/>
-      </c>
-      <c r="G138" s="45" t="str">
-        <f t="shared" si="64"/>
-        <v/>
-      </c>
-      <c r="H138" s="45" t="str">
-        <f t="shared" si="64"/>
-        <v/>
-      </c>
-    </row>
-    <row r="139" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B139" s="1" t="str">
-        <f t="shared" ref="B139:C139" si="65">IF(B97="","",B97)</f>
-        <v/>
-      </c>
-      <c r="C139" s="6" t="str">
-        <f t="shared" si="65"/>
-        <v/>
-      </c>
-      <c r="D139" s="44" t="str">
-        <f t="shared" ref="D139:H139" si="66">IF(D97="","",IF(D56="","-",(D97-D56)/D56))</f>
-        <v/>
-      </c>
-      <c r="E139" s="45" t="str">
-        <f t="shared" si="66"/>
-        <v/>
-      </c>
-      <c r="F139" s="45" t="str">
-        <f t="shared" si="66"/>
-        <v/>
-      </c>
-      <c r="G139" s="45" t="str">
-        <f t="shared" si="66"/>
-        <v/>
-      </c>
-      <c r="H139" s="45" t="str">
-        <f t="shared" si="66"/>
-        <v/>
-      </c>
-    </row>
-    <row r="140" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B140" s="1" t="str">
-        <f t="shared" ref="B140:C140" si="67">IF(B98="","",B98)</f>
-        <v/>
-      </c>
-      <c r="C140" s="6" t="str">
-        <f t="shared" si="67"/>
-        <v/>
-      </c>
-      <c r="D140" s="44" t="str">
-        <f t="shared" ref="D140:H140" si="68">IF(D98="","",IF(D57="","-",(D98-D57)/D57))</f>
-        <v/>
-      </c>
-      <c r="E140" s="45" t="str">
-        <f t="shared" si="68"/>
-        <v/>
-      </c>
-      <c r="F140" s="45" t="str">
-        <f t="shared" si="68"/>
-        <v/>
-      </c>
-      <c r="G140" s="45" t="str">
-        <f t="shared" si="68"/>
-        <v/>
-      </c>
-      <c r="H140" s="45" t="str">
-        <f t="shared" si="68"/>
-        <v/>
-      </c>
-    </row>
-    <row r="141" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B141" s="1" t="str">
-        <f t="shared" ref="B141:C141" si="69">IF(B99="","",B99)</f>
-        <v/>
-      </c>
-      <c r="C141" s="6" t="str">
-        <f t="shared" si="69"/>
-        <v/>
-      </c>
-      <c r="D141" s="44" t="str">
-        <f t="shared" ref="D141:H141" si="70">IF(D99="","",IF(D58="","-",(D99-D58)/D58))</f>
-        <v/>
-      </c>
-      <c r="E141" s="45" t="str">
-        <f t="shared" si="70"/>
-        <v/>
-      </c>
-      <c r="F141" s="45" t="str">
-        <f t="shared" si="70"/>
-        <v/>
-      </c>
-      <c r="G141" s="45" t="str">
-        <f t="shared" si="70"/>
-        <v/>
-      </c>
-      <c r="H141" s="45" t="str">
-        <f t="shared" si="70"/>
-        <v/>
-      </c>
-    </row>
-    <row r="142" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B142" s="1" t="str">
-        <f t="shared" ref="B142:C142" si="71">IF(B100="","",B100)</f>
-        <v/>
-      </c>
-      <c r="C142" s="6" t="str">
-        <f t="shared" si="71"/>
-        <v/>
-      </c>
-      <c r="D142" s="44" t="str">
-        <f t="shared" ref="D142:H142" si="72">IF(D100="","",IF(D59="","-",(D100-D59)/D59))</f>
-        <v/>
-      </c>
-      <c r="E142" s="45" t="str">
-        <f t="shared" si="72"/>
-        <v/>
-      </c>
-      <c r="F142" s="45" t="str">
-        <f t="shared" si="72"/>
-        <v/>
-      </c>
-      <c r="G142" s="45" t="str">
-        <f t="shared" si="72"/>
-        <v/>
-      </c>
-      <c r="H142" s="45" t="str">
-        <f t="shared" si="72"/>
-        <v/>
-      </c>
+      <c r="D142" s="44"/>
+      <c r="E142" s="45"/>
+      <c r="F142" s="45"/>
+      <c r="G142" s="45"/>
+      <c r="H142" s="45"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
2190 - Remove the template formulas and align the cell map with the review
The template has no formulas: Comp prev difference labels and dates are
written by the writer. Filled posts totals and service types are one range
per table, and the short-term sheet uses the same layout as the others.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/_99_publication/monthly_tracker_filled_posts/templates/diagnostics_template.xlsx
+++ b/projects/_99_publication/monthly_tracker_filled_posts/templates/diagnostics_template.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{098FF929-F05E-4B79-9C37-493ECD078187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBC929C9-0AC8-44E6-A07F-B4EA6AC5970E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-885" windowWidth="29040" windowHeight="15720" tabRatio="779" xr2:uid="{E876E9E8-942E-455D-9B41-2B7C7CFBA90D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="779" activeTab="2" xr2:uid="{E876E9E8-942E-455D-9B41-2B7C7CFBA90D}"/>
   </bookViews>
   <sheets>
     <sheet name="Filled posts" sheetId="16" r:id="rId1"/>
@@ -414,7 +414,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -508,23 +508,13 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -5712,7 +5702,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Comp SfC and CT - short term'!$C$25</c:f>
+              <c:f>'Comp SfC and CT - short term'!$C$28</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5735,7 +5725,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$B$26:$B$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$B$29:$B$41</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
                 <c:ptCount val="13"/>
@@ -5744,7 +5734,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$C$26:$C$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$C$29:$C$41</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="13"/>
@@ -5763,7 +5753,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Comp SfC and CT - short term'!$D$25</c:f>
+              <c:f>'Comp SfC and CT - short term'!$D$28</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5786,7 +5776,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$B$26:$B$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$B$29:$B$41</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
                 <c:ptCount val="13"/>
@@ -5795,7 +5785,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$D$26:$D$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$D$29:$D$41</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="13"/>
@@ -6078,7 +6068,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Comp SfC and CT - short term'!$N$25</c:f>
+              <c:f>'Comp SfC and CT - short term'!$N$28</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6101,7 +6091,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$B$26:$B$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$B$29:$B$41</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
                 <c:ptCount val="13"/>
@@ -6110,7 +6100,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$N$26:$N$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$N$29:$N$41</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="13"/>
@@ -6129,7 +6119,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Comp SfC and CT - short term'!$O$25</c:f>
+              <c:f>'Comp SfC and CT - short term'!$O$28</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6152,7 +6142,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$B$26:$B$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$B$29:$B$41</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
                 <c:ptCount val="13"/>
@@ -6161,7 +6151,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$O$26:$O$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$O$29:$O$41</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="13"/>
@@ -6444,7 +6434,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Comp SfC and CT - short term'!$E$25</c:f>
+              <c:f>'Comp SfC and CT - short term'!$E$28</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6467,7 +6457,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$B$26:$B$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$B$29:$B$41</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
                 <c:ptCount val="13"/>
@@ -6476,7 +6466,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$E$26:$E$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$E$29:$E$41</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="13"/>
@@ -6495,7 +6485,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Comp SfC and CT - short term'!$F$25</c:f>
+              <c:f>'Comp SfC and CT - short term'!$F$28</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6518,7 +6508,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$B$26:$B$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$B$29:$B$41</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
                 <c:ptCount val="13"/>
@@ -6527,7 +6517,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$F$26:$F$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$F$29:$F$41</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="13"/>
@@ -6810,7 +6800,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Comp SfC and CT - short term'!$L$25</c:f>
+              <c:f>'Comp SfC and CT - short term'!$L$28</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6833,7 +6823,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$K$26:$K$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$K$29:$K$41</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
                 <c:ptCount val="13"/>
@@ -6842,7 +6832,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$L$26:$L$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$L$29:$L$41</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="13"/>
@@ -6861,7 +6851,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Comp SfC and CT - short term'!$M$25</c:f>
+              <c:f>'Comp SfC and CT - short term'!$M$28</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6884,7 +6874,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$K$26:$K$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$K$29:$K$41</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
                 <c:ptCount val="13"/>
@@ -6893,7 +6883,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Comp SfC and CT - short term'!$M$26:$M$38</c:f>
+              <c:f>'Comp SfC and CT - short term'!$M$29:$M$41</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="13"/>
@@ -18523,13 +18513,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>44824</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>44</xdr:row>
       <xdr:rowOff>33617</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>821031</xdr:colOff>
-      <xdr:row>55</xdr:row>
+      <xdr:row>58</xdr:row>
       <xdr:rowOff>66617</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -18561,13 +18551,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>44824</xdr:colOff>
-      <xdr:row>58</xdr:row>
+      <xdr:row>61</xdr:row>
       <xdr:rowOff>33617</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>115060</xdr:colOff>
-      <xdr:row>72</xdr:row>
+      <xdr:row>75</xdr:row>
       <xdr:rowOff>66617</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -18599,13 +18589,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>44824</xdr:colOff>
-      <xdr:row>58</xdr:row>
+      <xdr:row>61</xdr:row>
       <xdr:rowOff>33617</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>821031</xdr:colOff>
-      <xdr:row>72</xdr:row>
+      <xdr:row>75</xdr:row>
       <xdr:rowOff>66617</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -18637,13 +18627,13 @@
     <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>1098177</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>44</xdr:row>
       <xdr:rowOff>67235</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>36619</xdr:colOff>
-      <xdr:row>55</xdr:row>
+      <xdr:row>58</xdr:row>
       <xdr:rowOff>100235</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -23833,7 +23823,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53141A47-D662-4C6A-A262-AE56D00F283A}">
-  <dimension ref="B2:Z40"/>
+  <dimension ref="B2:Z43"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -24013,6 +24003,13 @@
       <c r="Z16" s="7"/>
     </row>
     <row r="17" spans="2:26" x14ac:dyDescent="0.2">
+      <c r="B17" s="63"/>
+      <c r="C17" s="63"/>
+      <c r="D17" s="63"/>
+      <c r="E17" s="63"/>
+      <c r="F17" s="63"/>
+      <c r="G17" s="63"/>
+      <c r="H17" s="63"/>
       <c r="N17" s="8"/>
       <c r="O17" s="7"/>
       <c r="U17" s="8"/>
@@ -24023,6 +24020,13 @@
       <c r="Z17" s="7"/>
     </row>
     <row r="18" spans="2:26" x14ac:dyDescent="0.2">
+      <c r="B18" s="63"/>
+      <c r="C18" s="63"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="63"/>
       <c r="N18" s="8"/>
       <c r="O18" s="7"/>
       <c r="U18" s="8"/>
@@ -24033,6 +24037,15 @@
       <c r="Z18" s="7"/>
     </row>
     <row r="19" spans="2:26" x14ac:dyDescent="0.2">
+      <c r="B19" s="63"/>
+      <c r="C19" s="63"/>
+      <c r="D19" s="63"/>
+      <c r="E19" s="63"/>
+      <c r="F19" s="63"/>
+      <c r="G19" s="63"/>
+      <c r="H19" s="63"/>
+      <c r="N19" s="8"/>
+      <c r="O19" s="7"/>
       <c r="U19" s="8"/>
       <c r="V19" s="8"/>
       <c r="W19" s="8"/>
@@ -24040,13 +24053,9 @@
       <c r="Y19" s="8"/>
       <c r="Z19" s="7"/>
     </row>
-    <row r="20" spans="2:26" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B20" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="K20" s="4" t="s">
-        <v>9</v>
-      </c>
+    <row r="20" spans="2:26" x14ac:dyDescent="0.2">
+      <c r="N20" s="8"/>
+      <c r="O20" s="7"/>
       <c r="U20" s="8"/>
       <c r="V20" s="8"/>
       <c r="W20" s="8"/>
@@ -24055,6 +24064,8 @@
       <c r="Z20" s="7"/>
     </row>
     <row r="21" spans="2:26" x14ac:dyDescent="0.2">
+      <c r="N21" s="8"/>
+      <c r="O21" s="7"/>
       <c r="U21" s="8"/>
       <c r="V21" s="8"/>
       <c r="W21" s="8"/>
@@ -24063,14 +24074,6 @@
       <c r="Z21" s="7"/>
     </row>
     <row r="22" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="B22" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D22" s="8"/>
-      <c r="K22" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M22" s="8"/>
       <c r="U22" s="8"/>
       <c r="V22" s="8"/>
       <c r="W22" s="8"/>
@@ -24078,7 +24081,13 @@
       <c r="Y22" s="8"/>
       <c r="Z22" s="7"/>
     </row>
-    <row r="23" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:26" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B23" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="U23" s="8"/>
       <c r="V23" s="8"/>
       <c r="W23" s="8"/>
@@ -24087,18 +24096,6 @@
       <c r="Z23" s="7"/>
     </row>
     <row r="24" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="C24" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="D24" s="14"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="14"/>
-      <c r="L24" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="M24" s="14"/>
-      <c r="N24" s="13"/>
-      <c r="O24" s="14"/>
       <c r="U24" s="8"/>
       <c r="V24" s="8"/>
       <c r="W24" s="8"/>
@@ -24106,31 +24103,15 @@
       <c r="Y24" s="8"/>
       <c r="Z24" s="7"/>
     </row>
-    <row r="25" spans="2:26" ht="30" x14ac:dyDescent="0.2">
-      <c r="C25" s="20" t="s">
-        <v>20</v>
+    <row r="25" spans="2:26" x14ac:dyDescent="0.2">
+      <c r="B25" s="1" t="s">
+        <v>19</v>
       </c>
-      <c r="D25" s="17" t="s">
-        <v>21</v>
+      <c r="D25" s="8"/>
+      <c r="K25" s="1" t="s">
+        <v>19</v>
       </c>
-      <c r="E25" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="F25" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="L25" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="M25" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="N25" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="O25" s="17" t="s">
-        <v>21</v>
-      </c>
+      <c r="M25" s="8"/>
       <c r="U25" s="8"/>
       <c r="V25" s="8"/>
       <c r="W25" s="8"/>
@@ -24139,52 +24120,76 @@
       <c r="Z25" s="7"/>
     </row>
     <row r="26" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="B26" s="18"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="26"/>
-      <c r="K26" s="18"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="42"/>
-      <c r="N26" s="25"/>
-      <c r="O26" s="26"/>
+      <c r="U26" s="8"/>
+      <c r="V26" s="8"/>
+      <c r="W26" s="8"/>
+      <c r="X26" s="7"/>
+      <c r="Y26" s="8"/>
+      <c r="Z26" s="7"/>
     </row>
     <row r="27" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="B27" s="6"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="28"/>
-      <c r="F27" s="12"/>
-      <c r="K27" s="6"/>
-      <c r="L27" s="15"/>
-      <c r="M27" s="8"/>
-      <c r="N27" s="28"/>
-      <c r="O27" s="12"/>
-    </row>
-    <row r="28" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="B28" s="6"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="12"/>
-      <c r="K28" s="6"/>
-      <c r="L28" s="15"/>
-      <c r="M28" s="8"/>
-      <c r="N28" s="28"/>
-      <c r="O28" s="12"/>
+      <c r="C27" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27" s="14"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="14"/>
+      <c r="L27" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="M27" s="14"/>
+      <c r="N27" s="13"/>
+      <c r="O27" s="14"/>
+      <c r="U27" s="8"/>
+      <c r="V27" s="8"/>
+      <c r="W27" s="8"/>
+      <c r="X27" s="7"/>
+      <c r="Y27" s="8"/>
+      <c r="Z27" s="7"/>
+    </row>
+    <row r="28" spans="2:26" ht="30" x14ac:dyDescent="0.2">
+      <c r="C28" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="E28" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="L28" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="M28" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="N28" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="O28" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="U28" s="8"/>
+      <c r="V28" s="8"/>
+      <c r="W28" s="8"/>
+      <c r="X28" s="7"/>
+      <c r="Y28" s="8"/>
+      <c r="Z28" s="7"/>
     </row>
     <row r="29" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="B29" s="6"/>
-      <c r="C29" s="15"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="12"/>
-      <c r="K29" s="6"/>
-      <c r="L29" s="15"/>
-      <c r="M29" s="8"/>
-      <c r="N29" s="28"/>
-      <c r="O29" s="12"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="42"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="26"/>
+      <c r="K29" s="18"/>
+      <c r="L29" s="16"/>
+      <c r="M29" s="42"/>
+      <c r="N29" s="25"/>
+      <c r="O29" s="26"/>
     </row>
     <row r="30" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B30" s="6"/>
@@ -24294,29 +24299,65 @@
       <c r="N38" s="28"/>
       <c r="O38" s="12"/>
     </row>
-    <row r="39" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B39" s="6"/>
-      <c r="C39" s="8"/>
+      <c r="C39" s="15"/>
       <c r="D39" s="8"/>
-      <c r="E39" s="3"/>
-      <c r="F39" s="3"/>
+      <c r="E39" s="28"/>
+      <c r="F39" s="12"/>
       <c r="K39" s="6"/>
-      <c r="L39" s="8"/>
+      <c r="L39" s="15"/>
       <c r="M39" s="8"/>
-      <c r="N39" s="3"/>
-      <c r="O39" s="3"/>
-    </row>
-    <row r="40" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="N39" s="28"/>
+      <c r="O39" s="12"/>
+    </row>
+    <row r="40" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B40" s="6"/>
-      <c r="C40" s="8"/>
+      <c r="C40" s="15"/>
       <c r="D40" s="8"/>
-      <c r="E40" s="3"/>
-      <c r="F40" s="3"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="12"/>
       <c r="K40" s="6"/>
-      <c r="L40" s="8"/>
+      <c r="L40" s="15"/>
       <c r="M40" s="8"/>
-      <c r="N40" s="3"/>
-      <c r="O40" s="3"/>
+      <c r="N40" s="28"/>
+      <c r="O40" s="12"/>
+    </row>
+    <row r="41" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B41" s="6"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="28"/>
+      <c r="F41" s="12"/>
+      <c r="K41" s="6"/>
+      <c r="L41" s="15"/>
+      <c r="M41" s="8"/>
+      <c r="N41" s="28"/>
+      <c r="O41" s="12"/>
+    </row>
+    <row r="42" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B42" s="6"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="K42" s="6"/>
+      <c r="L42" s="8"/>
+      <c r="M42" s="8"/>
+      <c r="N42" s="3"/>
+      <c r="O42" s="3"/>
+    </row>
+    <row r="43" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B43" s="6"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="K43" s="6"/>
+      <c r="L43" s="8"/>
+      <c r="M43" s="8"/>
+      <c r="N43" s="3"/>
+      <c r="O43" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
2190 - Clear the Comp prev difference formulas from the template
Opens on Filled posts with A1 selected on every tab; document metadata stripped.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/_99_publication/monthly_tracker_filled_posts/templates/diagnostics_template.xlsx
+++ b/projects/_99_publication/monthly_tracker_filled_posts/templates/diagnostics_template.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBC929C9-0AC8-44E6-A07F-B4EA6AC5970E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC569A31-188A-4187-B9E5-78F342640612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="779" activeTab="2" xr2:uid="{E876E9E8-942E-455D-9B41-2B7C7CFBA90D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="779" xr2:uid="{E876E9E8-942E-455D-9B41-2B7C7CFBA90D}"/>
   </bookViews>
   <sheets>
     <sheet name="Filled posts" sheetId="16" r:id="rId1"/>
@@ -414,7 +414,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -508,7 +508,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -23262,14 +23261,8 @@
       </c>
     </row>
     <row r="106" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B106" s="43" t="str">
-        <f>IF(B64="","",B64)</f>
-        <v/>
-      </c>
-      <c r="C106" s="6" t="str">
-        <f>IF(C64="","",C64)</f>
-        <v/>
-      </c>
+      <c r="B106" s="43"/>
+      <c r="C106" s="6"/>
       <c r="D106" s="25"/>
       <c r="E106" s="26"/>
       <c r="F106" s="26"/>
@@ -23277,14 +23270,7 @@
       <c r="H106" s="26"/>
     </row>
     <row r="107" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B107" s="1" t="str">
-        <f t="shared" ref="B107:C107" si="0">IF(B65="","",B65)</f>
-        <v/>
-      </c>
-      <c r="C107" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
+      <c r="C107" s="6"/>
       <c r="D107" s="28"/>
       <c r="E107" s="12"/>
       <c r="F107" s="12"/>
@@ -23292,14 +23278,7 @@
       <c r="H107" s="12"/>
     </row>
     <row r="108" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B108" s="1" t="str">
-        <f t="shared" ref="B108:C108" si="1">IF(B66="","",B66)</f>
-        <v/>
-      </c>
-      <c r="C108" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="C108" s="6"/>
       <c r="D108" s="28"/>
       <c r="E108" s="12"/>
       <c r="F108" s="12"/>
@@ -23307,14 +23286,7 @@
       <c r="H108" s="12"/>
     </row>
     <row r="109" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B109" s="1" t="str">
-        <f t="shared" ref="B109:C109" si="2">IF(B67="","",B67)</f>
-        <v/>
-      </c>
-      <c r="C109" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
+      <c r="C109" s="6"/>
       <c r="D109" s="28"/>
       <c r="E109" s="12"/>
       <c r="F109" s="12"/>
@@ -23322,14 +23294,7 @@
       <c r="H109" s="12"/>
     </row>
     <row r="110" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B110" s="1" t="str">
-        <f t="shared" ref="B110:C110" si="3">IF(B68="","",B68)</f>
-        <v/>
-      </c>
-      <c r="C110" s="6" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="C110" s="6"/>
       <c r="D110" s="28"/>
       <c r="E110" s="12"/>
       <c r="F110" s="12"/>
@@ -23337,14 +23302,7 @@
       <c r="H110" s="12"/>
     </row>
     <row r="111" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B111" s="1" t="str">
-        <f t="shared" ref="B111:C111" si="4">IF(B69="","",B69)</f>
-        <v/>
-      </c>
-      <c r="C111" s="6" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
+      <c r="C111" s="6"/>
       <c r="D111" s="28"/>
       <c r="E111" s="12"/>
       <c r="F111" s="12"/>
@@ -23352,464 +23310,247 @@
       <c r="H111" s="12"/>
     </row>
     <row r="112" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B112" s="1" t="str">
-        <f t="shared" ref="B112:C112" si="5">IF(B70="","",B70)</f>
-        <v/>
-      </c>
-      <c r="C112" s="6" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
+      <c r="C112" s="6"/>
       <c r="D112" s="28"/>
       <c r="E112" s="12"/>
       <c r="F112" s="12"/>
       <c r="G112" s="12"/>
       <c r="H112" s="12"/>
     </row>
-    <row r="113" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B113" s="1" t="str">
-        <f t="shared" ref="B113:C113" si="6">IF(B71="","",B71)</f>
-        <v/>
-      </c>
-      <c r="C113" s="6" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
+    <row r="113" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C113" s="6"/>
       <c r="D113" s="28"/>
       <c r="E113" s="12"/>
       <c r="F113" s="12"/>
       <c r="G113" s="12"/>
       <c r="H113" s="12"/>
     </row>
-    <row r="114" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B114" s="1" t="str">
-        <f t="shared" ref="B114:C114" si="7">IF(B72="","",B72)</f>
-        <v/>
-      </c>
-      <c r="C114" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
+    <row r="114" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C114" s="6"/>
       <c r="D114" s="28"/>
       <c r="E114" s="12"/>
       <c r="F114" s="12"/>
       <c r="G114" s="12"/>
       <c r="H114" s="12"/>
     </row>
-    <row r="115" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B115" s="1" t="str">
-        <f t="shared" ref="B115:C115" si="8">IF(B73="","",B73)</f>
-        <v/>
-      </c>
-      <c r="C115" s="6" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
+    <row r="115" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C115" s="6"/>
       <c r="D115" s="28"/>
       <c r="E115" s="12"/>
       <c r="F115" s="12"/>
       <c r="G115" s="12"/>
       <c r="H115" s="12"/>
     </row>
-    <row r="116" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B116" s="1" t="str">
-        <f t="shared" ref="B116:C116" si="9">IF(B74="","",B74)</f>
-        <v/>
-      </c>
-      <c r="C116" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
+    <row r="116" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C116" s="6"/>
       <c r="D116" s="28"/>
       <c r="E116" s="12"/>
       <c r="F116" s="12"/>
       <c r="G116" s="12"/>
       <c r="H116" s="12"/>
     </row>
-    <row r="117" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B117" s="1" t="str">
-        <f t="shared" ref="B117:C117" si="10">IF(B75="","",B75)</f>
-        <v/>
-      </c>
-      <c r="C117" s="6" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
+    <row r="117" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C117" s="6"/>
       <c r="D117" s="28"/>
       <c r="E117" s="12"/>
       <c r="F117" s="12"/>
       <c r="G117" s="12"/>
       <c r="H117" s="12"/>
     </row>
-    <row r="118" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B118" s="1" t="str">
-        <f t="shared" ref="B118:C118" si="11">IF(B76="","",B76)</f>
-        <v/>
-      </c>
-      <c r="C118" s="6" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
+    <row r="118" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C118" s="6"/>
       <c r="D118" s="28"/>
       <c r="E118" s="12"/>
       <c r="F118" s="12"/>
       <c r="G118" s="12"/>
       <c r="H118" s="12"/>
     </row>
-    <row r="119" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B119" s="1" t="str">
-        <f t="shared" ref="B119:C119" si="12">IF(B77="","",B77)</f>
-        <v/>
-      </c>
-      <c r="C119" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
+    <row r="119" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C119" s="6"/>
       <c r="D119" s="28"/>
       <c r="E119" s="12"/>
       <c r="F119" s="12"/>
       <c r="G119" s="12"/>
       <c r="H119" s="12"/>
     </row>
-    <row r="120" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B120" s="1" t="str">
-        <f t="shared" ref="B120:C120" si="13">IF(B78="","",B78)</f>
-        <v/>
-      </c>
-      <c r="C120" s="6" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
+    <row r="120" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C120" s="6"/>
       <c r="D120" s="28"/>
       <c r="E120" s="12"/>
       <c r="F120" s="12"/>
       <c r="G120" s="12"/>
       <c r="H120" s="12"/>
     </row>
-    <row r="121" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B121" s="1" t="str">
-        <f t="shared" ref="B121:C121" si="14">IF(B79="","",B79)</f>
-        <v/>
-      </c>
-      <c r="C121" s="6" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
+    <row r="121" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C121" s="6"/>
       <c r="D121" s="28"/>
       <c r="E121" s="12"/>
       <c r="F121" s="12"/>
       <c r="G121" s="12"/>
       <c r="H121" s="12"/>
     </row>
-    <row r="122" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B122" s="1" t="str">
-        <f t="shared" ref="B122:C122" si="15">IF(B80="","",B80)</f>
-        <v/>
-      </c>
-      <c r="C122" s="6" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
+    <row r="122" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C122" s="6"/>
       <c r="D122" s="28"/>
       <c r="E122" s="12"/>
       <c r="F122" s="12"/>
       <c r="G122" s="12"/>
       <c r="H122" s="12"/>
     </row>
-    <row r="123" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B123" s="1" t="str">
-        <f t="shared" ref="B123:C123" si="16">IF(B81="","",B81)</f>
-        <v/>
-      </c>
-      <c r="C123" s="6" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
+    <row r="123" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C123" s="6"/>
       <c r="D123" s="28"/>
       <c r="E123" s="12"/>
       <c r="F123" s="12"/>
       <c r="G123" s="12"/>
       <c r="H123" s="12"/>
     </row>
-    <row r="124" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B124" s="1" t="str">
-        <f t="shared" ref="B124:C124" si="17">IF(B82="","",B82)</f>
-        <v/>
-      </c>
-      <c r="C124" s="6" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
+    <row r="124" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C124" s="6"/>
       <c r="D124" s="28"/>
       <c r="E124" s="12"/>
       <c r="F124" s="12"/>
       <c r="G124" s="12"/>
       <c r="H124" s="12"/>
     </row>
-    <row r="125" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B125" s="1" t="str">
-        <f t="shared" ref="B125:C125" si="18">IF(B83="","",B83)</f>
-        <v/>
-      </c>
-      <c r="C125" s="6" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
+    <row r="125" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C125" s="6"/>
       <c r="D125" s="28"/>
       <c r="E125" s="12"/>
       <c r="F125" s="12"/>
       <c r="G125" s="12"/>
       <c r="H125" s="12"/>
     </row>
-    <row r="126" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B126" s="1" t="str">
-        <f t="shared" ref="B126:C126" si="19">IF(B84="","",B84)</f>
-        <v/>
-      </c>
-      <c r="C126" s="6" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
+    <row r="126" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C126" s="6"/>
       <c r="D126" s="28"/>
       <c r="E126" s="12"/>
       <c r="F126" s="12"/>
       <c r="G126" s="12"/>
       <c r="H126" s="12"/>
     </row>
-    <row r="127" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B127" s="1" t="str">
-        <f t="shared" ref="B127:C127" si="20">IF(B85="","",B85)</f>
-        <v/>
-      </c>
-      <c r="C127" s="6" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
+    <row r="127" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C127" s="6"/>
       <c r="D127" s="28"/>
       <c r="E127" s="12"/>
       <c r="F127" s="12"/>
       <c r="G127" s="12"/>
       <c r="H127" s="12"/>
     </row>
-    <row r="128" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B128" s="1" t="str">
-        <f t="shared" ref="B128:C128" si="21">IF(B86="","",B86)</f>
-        <v/>
-      </c>
-      <c r="C128" s="6" t="str">
-        <f t="shared" si="21"/>
-        <v/>
-      </c>
+    <row r="128" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C128" s="6"/>
       <c r="D128" s="28"/>
       <c r="E128" s="12"/>
       <c r="F128" s="12"/>
       <c r="G128" s="12"/>
       <c r="H128" s="12"/>
     </row>
-    <row r="129" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B129" s="1" t="str">
-        <f t="shared" ref="B129:C129" si="22">IF(B87="","",B87)</f>
-        <v/>
-      </c>
-      <c r="C129" s="6" t="str">
-        <f t="shared" si="22"/>
-        <v/>
-      </c>
+    <row r="129" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C129" s="6"/>
       <c r="D129" s="28"/>
       <c r="E129" s="12"/>
       <c r="F129" s="12"/>
       <c r="G129" s="12"/>
       <c r="H129" s="12"/>
     </row>
-    <row r="130" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B130" s="1" t="str">
-        <f t="shared" ref="B130:C130" si="23">IF(B88="","",B88)</f>
-        <v/>
-      </c>
-      <c r="C130" s="6" t="str">
-        <f t="shared" si="23"/>
-        <v/>
-      </c>
+    <row r="130" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C130" s="6"/>
       <c r="D130" s="28"/>
       <c r="E130" s="12"/>
       <c r="F130" s="12"/>
       <c r="G130" s="12"/>
       <c r="H130" s="12"/>
     </row>
-    <row r="131" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B131" s="1" t="str">
-        <f t="shared" ref="B131:C131" si="24">IF(B89="","",B89)</f>
-        <v/>
-      </c>
-      <c r="C131" s="6" t="str">
-        <f t="shared" si="24"/>
-        <v/>
-      </c>
+    <row r="131" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C131" s="6"/>
       <c r="D131" s="44"/>
       <c r="E131" s="45"/>
       <c r="F131" s="45"/>
       <c r="G131" s="45"/>
       <c r="H131" s="45"/>
     </row>
-    <row r="132" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B132" s="1" t="str">
-        <f t="shared" ref="B132:C132" si="25">IF(B90="","",B90)</f>
-        <v/>
-      </c>
-      <c r="C132" s="6" t="str">
-        <f t="shared" si="25"/>
-        <v/>
-      </c>
+    <row r="132" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C132" s="6"/>
       <c r="D132" s="44"/>
       <c r="E132" s="45"/>
       <c r="F132" s="45"/>
       <c r="G132" s="45"/>
       <c r="H132" s="45"/>
     </row>
-    <row r="133" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B133" s="1" t="str">
-        <f t="shared" ref="B133:C133" si="26">IF(B91="","",B91)</f>
-        <v/>
-      </c>
-      <c r="C133" s="6" t="str">
-        <f t="shared" si="26"/>
-        <v/>
-      </c>
+    <row r="133" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C133" s="6"/>
       <c r="D133" s="44"/>
       <c r="E133" s="45"/>
       <c r="F133" s="45"/>
       <c r="G133" s="45"/>
       <c r="H133" s="45"/>
     </row>
-    <row r="134" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B134" s="1" t="str">
-        <f t="shared" ref="B134:C134" si="27">IF(B92="","",B92)</f>
-        <v/>
-      </c>
-      <c r="C134" s="6" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
+    <row r="134" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C134" s="6"/>
       <c r="D134" s="44"/>
       <c r="E134" s="45"/>
       <c r="F134" s="45"/>
       <c r="G134" s="45"/>
       <c r="H134" s="45"/>
     </row>
-    <row r="135" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B135" s="1" t="str">
-        <f t="shared" ref="B135:C135" si="28">IF(B93="","",B93)</f>
-        <v/>
-      </c>
-      <c r="C135" s="6" t="str">
-        <f t="shared" si="28"/>
-        <v/>
-      </c>
+    <row r="135" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C135" s="6"/>
       <c r="D135" s="44"/>
       <c r="E135" s="45"/>
       <c r="F135" s="45"/>
       <c r="G135" s="45"/>
       <c r="H135" s="45"/>
     </row>
-    <row r="136" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B136" s="1" t="str">
-        <f t="shared" ref="B136:C136" si="29">IF(B94="","",B94)</f>
-        <v/>
-      </c>
-      <c r="C136" s="6" t="str">
-        <f t="shared" si="29"/>
-        <v/>
-      </c>
+    <row r="136" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C136" s="6"/>
       <c r="D136" s="44"/>
       <c r="E136" s="45"/>
       <c r="F136" s="45"/>
       <c r="G136" s="45"/>
       <c r="H136" s="45"/>
     </row>
-    <row r="137" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B137" s="1" t="str">
-        <f t="shared" ref="B137:C137" si="30">IF(B95="","",B95)</f>
-        <v/>
-      </c>
-      <c r="C137" s="6" t="str">
-        <f t="shared" si="30"/>
-        <v/>
-      </c>
+    <row r="137" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C137" s="6"/>
       <c r="D137" s="44"/>
       <c r="E137" s="45"/>
       <c r="F137" s="45"/>
       <c r="G137" s="45"/>
       <c r="H137" s="45"/>
     </row>
-    <row r="138" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B138" s="1" t="str">
-        <f t="shared" ref="B138:C138" si="31">IF(B96="","",B96)</f>
-        <v/>
-      </c>
-      <c r="C138" s="6" t="str">
-        <f t="shared" si="31"/>
-        <v/>
-      </c>
+    <row r="138" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C138" s="6"/>
       <c r="D138" s="44"/>
       <c r="E138" s="45"/>
       <c r="F138" s="45"/>
       <c r="G138" s="45"/>
       <c r="H138" s="45"/>
     </row>
-    <row r="139" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B139" s="1" t="str">
-        <f t="shared" ref="B139:C139" si="32">IF(B97="","",B97)</f>
-        <v/>
-      </c>
-      <c r="C139" s="6" t="str">
-        <f t="shared" si="32"/>
-        <v/>
-      </c>
+    <row r="139" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C139" s="6"/>
       <c r="D139" s="44"/>
       <c r="E139" s="45"/>
       <c r="F139" s="45"/>
       <c r="G139" s="45"/>
       <c r="H139" s="45"/>
     </row>
-    <row r="140" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B140" s="1" t="str">
-        <f t="shared" ref="B140:C140" si="33">IF(B98="","",B98)</f>
-        <v/>
-      </c>
-      <c r="C140" s="6" t="str">
-        <f t="shared" si="33"/>
-        <v/>
-      </c>
+    <row r="140" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C140" s="6"/>
       <c r="D140" s="44"/>
       <c r="E140" s="45"/>
       <c r="F140" s="45"/>
       <c r="G140" s="45"/>
       <c r="H140" s="45"/>
     </row>
-    <row r="141" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B141" s="1" t="str">
-        <f t="shared" ref="B141:C141" si="34">IF(B99="","",B99)</f>
-        <v/>
-      </c>
-      <c r="C141" s="6" t="str">
-        <f t="shared" si="34"/>
-        <v/>
-      </c>
+    <row r="141" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C141" s="6"/>
       <c r="D141" s="44"/>
       <c r="E141" s="45"/>
       <c r="F141" s="45"/>
       <c r="G141" s="45"/>
       <c r="H141" s="45"/>
     </row>
-    <row r="142" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B142" s="1" t="str">
-        <f t="shared" ref="B142:C142" si="35">IF(B100="","",B100)</f>
-        <v/>
-      </c>
-      <c r="C142" s="6" t="str">
-        <f t="shared" si="35"/>
-        <v/>
-      </c>
+    <row r="142" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C142" s="6"/>
       <c r="D142" s="44"/>
       <c r="E142" s="45"/>
       <c r="F142" s="45"/>
@@ -24003,13 +23744,6 @@
       <c r="Z16" s="7"/>
     </row>
     <row r="17" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="B17" s="63"/>
-      <c r="C17" s="63"/>
-      <c r="D17" s="63"/>
-      <c r="E17" s="63"/>
-      <c r="F17" s="63"/>
-      <c r="G17" s="63"/>
-      <c r="H17" s="63"/>
       <c r="N17" s="8"/>
       <c r="O17" s="7"/>
       <c r="U17" s="8"/>
@@ -24020,13 +23754,6 @@
       <c r="Z17" s="7"/>
     </row>
     <row r="18" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="B18" s="63"/>
-      <c r="C18" s="63"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
-      <c r="G18" s="63"/>
-      <c r="H18" s="63"/>
       <c r="N18" s="8"/>
       <c r="O18" s="7"/>
       <c r="U18" s="8"/>
@@ -24037,13 +23764,6 @@
       <c r="Z18" s="7"/>
     </row>
     <row r="19" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="B19" s="63"/>
-      <c r="C19" s="63"/>
-      <c r="D19" s="63"/>
-      <c r="E19" s="63"/>
-      <c r="F19" s="63"/>
-      <c r="G19" s="63"/>
-      <c r="H19" s="63"/>
       <c r="N19" s="8"/>
       <c r="O19" s="7"/>
       <c r="U19" s="8"/>

</xml_diff>